<commit_message>
Update Dataset_inf.xlsx to match renamed studies
</commit_message>
<xml_diff>
--- a/1_Data/Dataset_inf.xlsx
+++ b/1_Data/Dataset_inf.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11028"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11028"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/T3/Dell5510/HCP_cloud/My_Lab/Projects/SPE_Database/1_Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D349CC3E-223A-5B40-9D8B-6354D0874423}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F43C018-C2EE-E646-9C67-27457FED6E61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="32260" yWindow="2540" windowWidth="32660" windowHeight="13940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1390" uniqueCount="517">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1391" uniqueCount="516">
   <si>
     <t>Note</t>
   </si>
@@ -249,27 +248,7 @@
     <t>Switch Identity: (Partner, Stranger)</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>1 (non-switch)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>; 2 (switched)</t>
-    </r>
+    <t>1 (non-switch); 2 (switched)</t>
   </si>
   <si>
     <t>United Kingdom</t>
@@ -519,7 +498,7 @@
     <t>2(matching condition: matching, mismatching) × 3(identity: self, stranger, celebrity) × 4(mood: happiness, anxiety, serenity, depression)</t>
   </si>
   <si>
-    <t>Qian_2019_QJEP</t>
+    <t>Qian_2020_QJEP</t>
   </si>
   <si>
     <t>https://osf.io/bw27c</t>
@@ -531,37 +510,7 @@
     <t>Celebrity</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Cue: (With; </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Without</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>)</t>
-    </r>
+    <t>Cue: (With; Without)</t>
   </si>
   <si>
     <t>2(identity:self,celebrity)*2(alertingcue:with,without)</t>
@@ -684,37 +633,7 @@
     <t>Golubickis &amp; Macrae</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Presentation: (</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Mixed</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>, Blocked)</t>
-    </r>
+    <t>Presentation: (Mixed, Blocked)</t>
   </si>
   <si>
     <t>Plymouth</t>
@@ -918,33 +837,7 @@
     <t>Xu_2021_CP</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <charset val="134"/>
-      </rPr>
-      <t>The datasets generated during and/or analysed during the current study are available from the corresponding author on reason</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t>_x0002_</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <charset val="134"/>
-      </rPr>
-      <t>able request.</t>
-    </r>
+    <t>The datasets generated during and/or analysed during the current study are available from the corresponding author on reason_x0002_able request.</t>
   </si>
   <si>
     <t>Ps1E1</t>
@@ -1160,60 +1053,10 @@
     <t>Liang et al.</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>TMS (</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Pre</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>; Post)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>1 (before TMS)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>, 2 (after TMS)</t>
-    </r>
+    <t>TMS (Pre; Post)</t>
+  </si>
+  <si>
+    <t>1 (before TMS), 2 (after TMS)</t>
   </si>
   <si>
     <t>3(TMS group: LpSTS, DLPFC, sham) × 2(Matching condition: matching, nonmatching) × 3(Shape category: self, friend, stranger)</t>
@@ -1675,9 +1518,6 @@
     <t>Wozniak_2020_PLOS</t>
   </si>
   <si>
-    <t>http://osf.io/2q9w7.</t>
-  </si>
-  <si>
     <t>Pu8E1</t>
   </si>
   <si>
@@ -1741,20 +1581,20 @@
     <t>Yang_2021_CP</t>
   </si>
   <si>
-    <t>Liang_2021_HBM</t>
-  </si>
-  <si>
     <t>Pt5E1</t>
   </si>
   <si>
     <t>Pt5</t>
+  </si>
+  <si>
+    <t>http://osf.io/2q9w7</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1812,18 +1652,10 @@
       <charset val="134"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Arial"/>
-      <charset val="134"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="5">
@@ -1865,11 +1697,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1924,13 +1756,21 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1940,11 +1780,6 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <mruColors>
-      <color rgb="FFCCE4F1"/>
-    </mruColors>
-  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -2217,45 +2052,45 @@
   <dimension ref="A1:KJ77"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="7.83203125" customWidth="1"/>
-    <col min="3" max="3" width="13.33203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-    <col min="5" max="5" width="10.1640625" customWidth="1"/>
-    <col min="6" max="6" width="13.1640625" customWidth="1"/>
-    <col min="7" max="7" width="17.33203125" customWidth="1"/>
-    <col min="8" max="8" width="15.1640625" customWidth="1"/>
-    <col min="9" max="9" width="24.5" customWidth="1"/>
+    <col min="1" max="1" width="20" style="18" customWidth="1"/>
+    <col min="2" max="2" width="7.83203125" style="18" customWidth="1"/>
+    <col min="3" max="3" width="13.33203125" style="18" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" style="18" customWidth="1"/>
+    <col min="5" max="5" width="10.1640625" style="18" customWidth="1"/>
+    <col min="6" max="6" width="13.1640625" style="18" customWidth="1"/>
+    <col min="7" max="7" width="17.33203125" style="18" customWidth="1"/>
+    <col min="8" max="8" width="15.1640625" style="18" customWidth="1"/>
+    <col min="9" max="9" width="24.5" style="18" customWidth="1"/>
     <col min="10" max="10" width="40" style="2" customWidth="1"/>
     <col min="11" max="11" width="23.33203125" style="2" customWidth="1"/>
     <col min="12" max="12" width="9" style="2" customWidth="1"/>
     <col min="13" max="13" width="67" style="2" customWidth="1"/>
-    <col min="14" max="14" width="7.5" customWidth="1"/>
-    <col min="15" max="16" width="9" customWidth="1"/>
-    <col min="17" max="17" width="20" customWidth="1"/>
-    <col min="18" max="18" width="21.5" customWidth="1"/>
-    <col min="19" max="19" width="17.83203125" customWidth="1"/>
-    <col min="20" max="20" width="14.1640625" customWidth="1"/>
-    <col min="21" max="21" width="12.83203125" customWidth="1"/>
-    <col min="22" max="22" width="13.1640625" customWidth="1"/>
-    <col min="23" max="23" width="41.6640625" customWidth="1"/>
-    <col min="24" max="24" width="29" customWidth="1"/>
+    <col min="14" max="14" width="7.5" style="18" customWidth="1"/>
+    <col min="15" max="16" width="9" style="18" customWidth="1"/>
+    <col min="17" max="17" width="20" style="18" customWidth="1"/>
+    <col min="18" max="18" width="21.5" style="18" customWidth="1"/>
+    <col min="19" max="19" width="17.83203125" style="18" customWidth="1"/>
+    <col min="20" max="20" width="14.1640625" style="18" customWidth="1"/>
+    <col min="21" max="21" width="12.83203125" style="18" customWidth="1"/>
+    <col min="22" max="22" width="13.1640625" style="18" customWidth="1"/>
+    <col min="23" max="23" width="41.6640625" style="18" customWidth="1"/>
+    <col min="24" max="24" width="29" style="18" customWidth="1"/>
     <col min="25" max="25" width="28.33203125" style="5" customWidth="1"/>
-    <col min="26" max="26" width="14.5" customWidth="1"/>
-    <col min="27" max="27" width="17.5" customWidth="1"/>
-    <col min="28" max="28" width="14.5" customWidth="1"/>
-    <col min="29" max="29" width="11.6640625" customWidth="1"/>
-    <col min="30" max="30" width="11.1640625" customWidth="1"/>
-    <col min="31" max="31" width="12.83203125" customWidth="1"/>
-    <col min="32" max="32" width="12.6640625" customWidth="1"/>
-    <col min="33" max="33" width="7.5" customWidth="1"/>
-    <col min="34" max="34" width="132.1640625" customWidth="1"/>
-    <col min="35" max="36" width="25.6640625" customWidth="1"/>
-    <col min="37" max="37" width="73.83203125" customWidth="1"/>
-    <col min="38" max="38" width="68.6640625" customWidth="1"/>
+    <col min="26" max="26" width="14.5" style="18" customWidth="1"/>
+    <col min="27" max="27" width="17.5" style="18" customWidth="1"/>
+    <col min="28" max="28" width="14.5" style="18" customWidth="1"/>
+    <col min="29" max="29" width="11.6640625" style="18" customWidth="1"/>
+    <col min="30" max="30" width="11.1640625" style="18" customWidth="1"/>
+    <col min="31" max="31" width="12.83203125" style="18" customWidth="1"/>
+    <col min="32" max="32" width="12.6640625" style="18" customWidth="1"/>
+    <col min="33" max="33" width="7.5" style="18" customWidth="1"/>
+    <col min="34" max="34" width="132.1640625" style="18" customWidth="1"/>
+    <col min="35" max="36" width="25.6640625" style="18" customWidth="1"/>
+    <col min="37" max="37" width="73.83203125" style="18" customWidth="1"/>
+    <col min="38" max="38" width="68.6640625" style="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:296" s="2" customFormat="1" ht="16">
+    <row r="1" spans="1:296" s="2" customFormat="1" ht="16" customHeight="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -2369,7 +2204,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:296" ht="19">
+    <row r="2" spans="1:296" ht="19" customHeight="1">
       <c r="A2" s="3" t="s">
         <v>37</v>
       </c>
@@ -2394,19 +2229,19 @@
       <c r="H2" s="8">
         <v>0</v>
       </c>
-      <c r="I2" s="18" t="s">
+      <c r="I2" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="J2" s="20" t="s">
+      <c r="J2" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="K2" s="18" t="s">
+      <c r="K2" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="L2" s="18">
+      <c r="L2" s="19">
         <v>2019</v>
       </c>
-      <c r="M2" s="18" t="s">
+      <c r="M2" s="19" t="s">
         <v>44</v>
       </c>
       <c r="N2" s="3">
@@ -2738,7 +2573,7 @@
       <c r="KI2" s="3"/>
       <c r="KJ2" s="3"/>
     </row>
-    <row r="3" spans="1:296" ht="19">
+    <row r="3" spans="1:296" ht="19" customHeight="1">
       <c r="A3" s="3" t="s">
         <v>37</v>
       </c>
@@ -2763,11 +2598,11 @@
       <c r="H3" s="8">
         <v>0</v>
       </c>
-      <c r="I3" s="18"/>
+      <c r="I3" s="23"/>
       <c r="J3" s="20"/>
-      <c r="K3" s="18"/>
-      <c r="L3" s="18"/>
-      <c r="M3" s="18"/>
+      <c r="K3" s="20"/>
+      <c r="L3" s="20"/>
+      <c r="M3" s="20"/>
       <c r="N3" s="3">
         <v>2</v>
       </c>
@@ -3097,7 +2932,7 @@
       <c r="KI3" s="3"/>
       <c r="KJ3" s="3"/>
     </row>
-    <row r="4" spans="1:296" ht="19">
+    <row r="4" spans="1:296" ht="19" customHeight="1">
       <c r="A4" s="3" t="s">
         <v>37</v>
       </c>
@@ -3122,11 +2957,11 @@
       <c r="H4" s="8">
         <v>0</v>
       </c>
-      <c r="I4" s="18"/>
+      <c r="I4" s="23"/>
       <c r="J4" s="20"/>
-      <c r="K4" s="18"/>
-      <c r="L4" s="18"/>
-      <c r="M4" s="18"/>
+      <c r="K4" s="20"/>
+      <c r="L4" s="20"/>
+      <c r="M4" s="20"/>
       <c r="N4" s="3">
         <v>3</v>
       </c>
@@ -3456,7 +3291,7 @@
       <c r="KI4" s="3"/>
       <c r="KJ4" s="3"/>
     </row>
-    <row r="5" spans="1:296" ht="19">
+    <row r="5" spans="1:296" ht="19" customHeight="1">
       <c r="A5" s="3" t="s">
         <v>37</v>
       </c>
@@ -3481,11 +3316,11 @@
       <c r="H5" s="8">
         <v>0</v>
       </c>
-      <c r="I5" s="18"/>
+      <c r="I5" s="23"/>
       <c r="J5" s="20"/>
-      <c r="K5" s="18"/>
-      <c r="L5" s="18"/>
-      <c r="M5" s="18"/>
+      <c r="K5" s="20"/>
+      <c r="L5" s="20"/>
+      <c r="M5" s="20"/>
       <c r="N5" s="3">
         <v>4</v>
       </c>
@@ -4188,7 +4023,7 @@
       <c r="KI6" s="3"/>
       <c r="KJ6" s="3"/>
     </row>
-    <row r="7" spans="1:296" ht="19">
+    <row r="7" spans="1:296" ht="19" customHeight="1">
       <c r="A7" s="3"/>
       <c r="B7" s="3">
         <v>6</v>
@@ -4209,19 +4044,19 @@
       <c r="H7" s="8">
         <v>0</v>
       </c>
-      <c r="I7" s="18" t="s">
+      <c r="I7" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="J7" s="20" t="s">
+      <c r="J7" s="21" t="s">
         <v>79</v>
       </c>
-      <c r="K7" s="18" t="s">
+      <c r="K7" s="19" t="s">
         <v>80</v>
       </c>
-      <c r="L7" s="18">
+      <c r="L7" s="19">
         <v>2021</v>
       </c>
-      <c r="M7" s="18" t="s">
+      <c r="M7" s="19" t="s">
         <v>66</v>
       </c>
       <c r="N7" s="3">
@@ -4558,7 +4393,7 @@
       <c r="KI7" s="3"/>
       <c r="KJ7" s="3"/>
     </row>
-    <row r="8" spans="1:296" ht="19">
+    <row r="8" spans="1:296" ht="19" customHeight="1">
       <c r="A8" s="3"/>
       <c r="B8" s="3">
         <v>7</v>
@@ -4579,11 +4414,11 @@
       <c r="H8" s="8">
         <v>0</v>
       </c>
-      <c r="I8" s="18"/>
+      <c r="I8" s="23"/>
       <c r="J8" s="20"/>
-      <c r="K8" s="18"/>
-      <c r="L8" s="18"/>
-      <c r="M8" s="18"/>
+      <c r="K8" s="20"/>
+      <c r="L8" s="20"/>
+      <c r="M8" s="20"/>
       <c r="N8" s="3">
         <v>2</v>
       </c>
@@ -4898,7 +4733,7 @@
       <c r="KI8" s="3"/>
       <c r="KJ8" s="3"/>
     </row>
-    <row r="9" spans="1:296" ht="19">
+    <row r="9" spans="1:296" ht="19" customHeight="1">
       <c r="A9" s="3"/>
       <c r="B9" s="3">
         <v>8</v>
@@ -5263,7 +5098,7 @@
       <c r="KI9" s="3"/>
       <c r="KJ9" s="3"/>
     </row>
-    <row r="10" spans="1:296" ht="34">
+    <row r="10" spans="1:296" ht="34" customHeight="1">
       <c r="A10" t="s">
         <v>105</v>
       </c>
@@ -5630,7 +5465,7 @@
       <c r="KI10" s="3"/>
       <c r="KJ10" s="3"/>
     </row>
-    <row r="11" spans="1:296" ht="17">
+    <row r="11" spans="1:296" ht="17" customHeight="1">
       <c r="A11" s="3"/>
       <c r="B11" s="3">
         <v>10</v>
@@ -5996,7 +5831,7 @@
       <c r="KI11" s="3"/>
       <c r="KJ11" s="3"/>
     </row>
-    <row r="12" spans="1:296" ht="19">
+    <row r="12" spans="1:296" ht="19" customHeight="1">
       <c r="A12" s="3"/>
       <c r="B12" s="3">
         <v>11</v>
@@ -6017,19 +5852,19 @@
       <c r="H12" s="8">
         <v>0</v>
       </c>
-      <c r="I12" s="18" t="s">
+      <c r="I12" s="19" t="s">
         <v>134</v>
       </c>
-      <c r="J12" s="20" t="s">
+      <c r="J12" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="K12" s="18" t="s">
+      <c r="K12" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="L12" s="18">
+      <c r="L12" s="19">
         <v>2020</v>
       </c>
-      <c r="M12" s="18" t="s">
+      <c r="M12" s="19" t="s">
         <v>135</v>
       </c>
       <c r="N12" s="3">
@@ -6358,7 +6193,7 @@
       <c r="KI12" s="3"/>
       <c r="KJ12" s="3"/>
     </row>
-    <row r="13" spans="1:296" ht="19">
+    <row r="13" spans="1:296" ht="19" customHeight="1">
       <c r="A13" s="3"/>
       <c r="B13" s="3">
         <v>12</v>
@@ -6373,11 +6208,11 @@
       <c r="F13" s="7"/>
       <c r="G13" s="8"/>
       <c r="H13" s="8"/>
-      <c r="I13" s="18"/>
+      <c r="I13" s="23"/>
       <c r="J13" s="20"/>
-      <c r="K13" s="18"/>
-      <c r="L13" s="18"/>
-      <c r="M13" s="18"/>
+      <c r="K13" s="20"/>
+      <c r="L13" s="20"/>
+      <c r="M13" s="20"/>
       <c r="N13" s="3"/>
       <c r="O13" s="3"/>
       <c r="P13" s="3"/>
@@ -6686,7 +6521,7 @@
       <c r="KI13" s="3"/>
       <c r="KJ13" s="3"/>
     </row>
-    <row r="14" spans="1:296" ht="19">
+    <row r="14" spans="1:296" ht="19" customHeight="1">
       <c r="A14" s="3" t="s">
         <v>142</v>
       </c>
@@ -6711,19 +6546,19 @@
       <c r="H14" s="8">
         <v>0</v>
       </c>
-      <c r="I14" s="18" t="s">
+      <c r="I14" s="19" t="s">
         <v>145</v>
       </c>
-      <c r="J14" s="20" t="s">
+      <c r="J14" s="21" t="s">
         <v>146</v>
       </c>
-      <c r="K14" s="18" t="s">
+      <c r="K14" s="19" t="s">
         <v>147</v>
       </c>
-      <c r="L14" s="18">
+      <c r="L14" s="19">
         <v>2020</v>
       </c>
-      <c r="M14" s="18" t="s">
+      <c r="M14" s="19" t="s">
         <v>148</v>
       </c>
       <c r="N14" s="3">
@@ -7057,7 +6892,7 @@
       <c r="KI14" s="3"/>
       <c r="KJ14" s="3"/>
     </row>
-    <row r="15" spans="1:296" ht="19">
+    <row r="15" spans="1:296" ht="19" customHeight="1">
       <c r="A15" s="3"/>
       <c r="B15" s="3">
         <v>14</v>
@@ -7080,11 +6915,11 @@
       <c r="H15" s="8">
         <v>0</v>
       </c>
-      <c r="I15" s="18"/>
+      <c r="I15" s="23"/>
       <c r="J15" s="20"/>
-      <c r="K15" s="18"/>
-      <c r="L15" s="18"/>
-      <c r="M15" s="18"/>
+      <c r="K15" s="20"/>
+      <c r="L15" s="20"/>
+      <c r="M15" s="20"/>
       <c r="N15" s="3">
         <v>2</v>
       </c>
@@ -7416,7 +7251,7 @@
       <c r="KI15" s="3"/>
       <c r="KJ15" s="3"/>
     </row>
-    <row r="16" spans="1:296" ht="19">
+    <row r="16" spans="1:296" ht="19" customHeight="1">
       <c r="A16" s="3"/>
       <c r="B16" s="3">
         <v>15</v>
@@ -7439,19 +7274,19 @@
       <c r="H16" s="8">
         <v>0</v>
       </c>
-      <c r="I16" s="18" t="s">
+      <c r="I16" s="19" t="s">
         <v>161</v>
       </c>
-      <c r="J16" s="20" t="s">
+      <c r="J16" s="21" t="s">
         <v>162</v>
       </c>
-      <c r="K16" s="18" t="s">
+      <c r="K16" s="19" t="s">
         <v>163</v>
       </c>
-      <c r="L16" s="18">
+      <c r="L16" s="19">
         <v>2019</v>
       </c>
-      <c r="M16" s="18" t="s">
+      <c r="M16" s="19" t="s">
         <v>164</v>
       </c>
       <c r="N16" s="3">
@@ -7782,7 +7617,7 @@
       <c r="KI16" s="3"/>
       <c r="KJ16" s="3"/>
     </row>
-    <row r="17" spans="1:296" ht="19">
+    <row r="17" spans="1:296" ht="19" customHeight="1">
       <c r="A17" s="3"/>
       <c r="B17" s="3">
         <v>16</v>
@@ -7799,11 +7634,11 @@
       <c r="F17" s="7"/>
       <c r="G17" s="8"/>
       <c r="H17" s="7"/>
-      <c r="I17" s="18"/>
+      <c r="I17" s="23"/>
       <c r="J17" s="20"/>
-      <c r="K17" s="18"/>
-      <c r="L17" s="18"/>
-      <c r="M17" s="18"/>
+      <c r="K17" s="20"/>
+      <c r="L17" s="20"/>
+      <c r="M17" s="20"/>
       <c r="N17" s="3"/>
       <c r="O17" s="3"/>
       <c r="P17" s="3"/>
@@ -8113,7 +7948,7 @@
       <c r="KI17" s="3"/>
       <c r="KJ17" s="3"/>
     </row>
-    <row r="18" spans="1:296" ht="19">
+    <row r="18" spans="1:296" ht="19" customHeight="1">
       <c r="A18" s="3"/>
       <c r="B18" s="3">
         <v>17</v>
@@ -8130,11 +7965,11 @@
       <c r="F18" s="7"/>
       <c r="G18" s="8"/>
       <c r="H18" s="7"/>
-      <c r="I18" s="18"/>
+      <c r="I18" s="23"/>
       <c r="J18" s="20"/>
-      <c r="K18" s="18"/>
-      <c r="L18" s="18"/>
-      <c r="M18" s="18"/>
+      <c r="K18" s="20"/>
+      <c r="L18" s="20"/>
+      <c r="M18" s="20"/>
       <c r="N18" s="3"/>
       <c r="O18" s="3"/>
       <c r="P18" s="3"/>
@@ -8444,7 +8279,7 @@
       <c r="KI18" s="3"/>
       <c r="KJ18" s="3"/>
     </row>
-    <row r="19" spans="1:296" ht="19">
+    <row r="19" spans="1:296" ht="19" customHeight="1">
       <c r="A19" s="3" t="s">
         <v>178</v>
       </c>
@@ -8469,19 +8304,19 @@
       <c r="H19" s="7">
         <v>1</v>
       </c>
-      <c r="I19" s="18" t="s">
+      <c r="I19" s="19" t="s">
         <v>181</v>
       </c>
-      <c r="J19" s="20" t="s">
+      <c r="J19" s="21" t="s">
         <v>182</v>
       </c>
-      <c r="K19" s="18" t="s">
+      <c r="K19" s="19" t="s">
         <v>183</v>
       </c>
-      <c r="L19" s="18">
+      <c r="L19" s="19">
         <v>2018</v>
       </c>
-      <c r="M19" s="18" t="s">
+      <c r="M19" s="19" t="s">
         <v>184</v>
       </c>
       <c r="N19" s="3">
@@ -8540,7 +8375,7 @@
         <v>1</v>
       </c>
       <c r="AG19" s="3">
-        <f t="shared" ref="AG19:AG29" si="0">AC19-AF19</f>
+        <f t="shared" ref="AG19:AG54" si="0">AC19-AF19</f>
         <v>18</v>
       </c>
       <c r="AH19" s="3" t="s">
@@ -8816,7 +8651,7 @@
       <c r="KI19" s="3"/>
       <c r="KJ19" s="3"/>
     </row>
-    <row r="20" spans="1:296" ht="19">
+    <row r="20" spans="1:296" ht="19" customHeight="1">
       <c r="A20" s="3" t="s">
         <v>178</v>
       </c>
@@ -8841,11 +8676,11 @@
       <c r="H20" s="7">
         <v>1</v>
       </c>
-      <c r="I20" s="18"/>
+      <c r="I20" s="23"/>
       <c r="J20" s="20"/>
-      <c r="K20" s="18"/>
-      <c r="L20" s="18"/>
-      <c r="M20" s="18"/>
+      <c r="K20" s="20"/>
+      <c r="L20" s="20"/>
+      <c r="M20" s="20"/>
       <c r="N20" s="3">
         <v>2</v>
       </c>
@@ -9179,7 +9014,7 @@
       <c r="KI20" s="3"/>
       <c r="KJ20" s="3"/>
     </row>
-    <row r="21" spans="1:296" ht="19">
+    <row r="21" spans="1:296" ht="19" customHeight="1">
       <c r="A21" s="3" t="s">
         <v>192</v>
       </c>
@@ -9204,19 +9039,19 @@
       <c r="H21" s="8">
         <v>0</v>
       </c>
-      <c r="I21" s="18" t="s">
+      <c r="I21" s="19" t="s">
         <v>195</v>
       </c>
-      <c r="J21" s="20" t="s">
+      <c r="J21" s="21" t="s">
         <v>196</v>
       </c>
-      <c r="K21" s="18" t="s">
+      <c r="K21" s="19" t="s">
         <v>197</v>
       </c>
-      <c r="L21" s="18">
+      <c r="L21" s="19">
         <v>2021</v>
       </c>
-      <c r="M21" s="18" t="s">
+      <c r="M21" s="19" t="s">
         <v>66</v>
       </c>
       <c r="N21" s="3">
@@ -9550,7 +9385,7 @@
       <c r="KI21" s="3"/>
       <c r="KJ21" s="3"/>
     </row>
-    <row r="22" spans="1:296" ht="19">
+    <row r="22" spans="1:296" ht="19" customHeight="1">
       <c r="A22" s="3"/>
       <c r="B22" s="3">
         <v>21</v>
@@ -9573,11 +9408,11 @@
       <c r="H22" s="8">
         <v>0</v>
       </c>
-      <c r="I22" s="18"/>
+      <c r="I22" s="23"/>
       <c r="J22" s="20"/>
-      <c r="K22" s="18"/>
-      <c r="L22" s="18"/>
-      <c r="M22" s="18"/>
+      <c r="K22" s="20"/>
+      <c r="L22" s="20"/>
+      <c r="M22" s="20"/>
       <c r="N22" s="3">
         <v>2</v>
       </c>
@@ -9907,7 +9742,7 @@
       <c r="KI22" s="3"/>
       <c r="KJ22" s="3"/>
     </row>
-    <row r="23" spans="1:296" ht="19">
+    <row r="23" spans="1:296" ht="19" customHeight="1">
       <c r="A23" s="3"/>
       <c r="B23" s="3">
         <v>22</v>
@@ -9930,19 +9765,19 @@
       <c r="H23" s="8">
         <v>0</v>
       </c>
-      <c r="I23" s="18" t="s">
+      <c r="I23" s="19" t="s">
         <v>208</v>
       </c>
-      <c r="J23" s="20" t="s">
+      <c r="J23" s="21" t="s">
         <v>209</v>
       </c>
-      <c r="K23" s="18" t="s">
+      <c r="K23" s="19" t="s">
         <v>210</v>
       </c>
-      <c r="L23" s="18">
+      <c r="L23" s="19">
         <v>2021</v>
       </c>
-      <c r="M23" s="18" t="s">
+      <c r="M23" s="19" t="s">
         <v>66</v>
       </c>
       <c r="N23" s="3">
@@ -10276,7 +10111,7 @@
       <c r="KI23" s="3"/>
       <c r="KJ23" s="3"/>
     </row>
-    <row r="24" spans="1:296" ht="19">
+    <row r="24" spans="1:296" ht="19" customHeight="1">
       <c r="A24" s="3"/>
       <c r="B24" s="3">
         <v>23</v>
@@ -10299,11 +10134,11 @@
       <c r="H24" s="8">
         <v>0</v>
       </c>
-      <c r="I24" s="18"/>
+      <c r="I24" s="23"/>
       <c r="J24" s="20"/>
-      <c r="K24" s="18"/>
-      <c r="L24" s="18"/>
-      <c r="M24" s="18"/>
+      <c r="K24" s="20"/>
+      <c r="L24" s="20"/>
+      <c r="M24" s="20"/>
       <c r="N24" s="3">
         <v>2</v>
       </c>
@@ -10635,7 +10470,7 @@
       <c r="KI24" s="3"/>
       <c r="KJ24" s="3"/>
     </row>
-    <row r="25" spans="1:296" ht="19">
+    <row r="25" spans="1:296" ht="19" customHeight="1">
       <c r="A25" s="3"/>
       <c r="B25" s="3">
         <v>24</v>
@@ -10658,11 +10493,11 @@
       <c r="H25" s="8">
         <v>0</v>
       </c>
-      <c r="I25" s="18"/>
+      <c r="I25" s="23"/>
       <c r="J25" s="20"/>
-      <c r="K25" s="18"/>
-      <c r="L25" s="18"/>
-      <c r="M25" s="18"/>
+      <c r="K25" s="20"/>
+      <c r="L25" s="20"/>
+      <c r="M25" s="20"/>
       <c r="N25" s="3">
         <v>3</v>
       </c>
@@ -10994,7 +10829,7 @@
       <c r="KI25" s="3"/>
       <c r="KJ25" s="3"/>
     </row>
-    <row r="26" spans="1:296" ht="19">
+    <row r="26" spans="1:296" ht="19" customHeight="1">
       <c r="A26" s="3"/>
       <c r="B26" s="3">
         <v>25</v>
@@ -11017,11 +10852,11 @@
       <c r="H26" s="8">
         <v>0</v>
       </c>
-      <c r="I26" s="18"/>
+      <c r="I26" s="23"/>
       <c r="J26" s="20"/>
-      <c r="K26" s="18"/>
-      <c r="L26" s="18"/>
-      <c r="M26" s="18"/>
+      <c r="K26" s="20"/>
+      <c r="L26" s="20"/>
+      <c r="M26" s="20"/>
       <c r="N26" s="3">
         <v>4</v>
       </c>
@@ -11353,7 +11188,7 @@
       <c r="KI26" s="3"/>
       <c r="KJ26" s="3"/>
     </row>
-    <row r="27" spans="1:296" ht="16">
+    <row r="27" spans="1:296" ht="16" customHeight="1">
       <c r="A27" s="3"/>
       <c r="B27" s="3">
         <v>26</v>
@@ -11374,19 +11209,19 @@
       <c r="H27" s="8">
         <v>0</v>
       </c>
-      <c r="I27" s="18" t="s">
+      <c r="I27" s="19" t="s">
         <v>227</v>
       </c>
-      <c r="J27" s="20" t="s">
+      <c r="J27" s="21" t="s">
         <v>228</v>
       </c>
-      <c r="K27" s="18" t="s">
+      <c r="K27" s="19" t="s">
         <v>229</v>
       </c>
-      <c r="L27" s="18">
+      <c r="L27" s="19">
         <v>2020</v>
       </c>
-      <c r="M27" s="18" t="s">
+      <c r="M27" s="19" t="s">
         <v>230</v>
       </c>
       <c r="N27" s="3">
@@ -11718,7 +11553,7 @@
       <c r="KI27" s="3"/>
       <c r="KJ27" s="3"/>
     </row>
-    <row r="28" spans="1:296" ht="16">
+    <row r="28" spans="1:296" ht="16" customHeight="1">
       <c r="A28" s="3"/>
       <c r="B28" s="3">
         <v>27</v>
@@ -11739,11 +11574,11 @@
       <c r="H28" s="8">
         <v>0</v>
       </c>
-      <c r="I28" s="18"/>
+      <c r="I28" s="23"/>
       <c r="J28" s="20"/>
-      <c r="K28" s="18"/>
-      <c r="L28" s="18"/>
-      <c r="M28" s="18"/>
+      <c r="K28" s="20"/>
+      <c r="L28" s="20"/>
+      <c r="M28" s="20"/>
       <c r="N28" s="3">
         <v>2</v>
       </c>
@@ -12073,7 +11908,7 @@
       <c r="KI28" s="3"/>
       <c r="KJ28" s="3"/>
     </row>
-    <row r="29" spans="1:296" ht="16">
+    <row r="29" spans="1:296" ht="16" customHeight="1">
       <c r="A29" s="3"/>
       <c r="B29" s="3">
         <v>28</v>
@@ -12094,11 +11929,11 @@
       <c r="H29" s="8">
         <v>0</v>
       </c>
-      <c r="I29" s="18"/>
+      <c r="I29" s="23"/>
       <c r="J29" s="20"/>
-      <c r="K29" s="18"/>
-      <c r="L29" s="18"/>
-      <c r="M29" s="18"/>
+      <c r="K29" s="20"/>
+      <c r="L29" s="20"/>
+      <c r="M29" s="20"/>
       <c r="N29" s="3">
         <v>3</v>
       </c>
@@ -12428,7 +12263,7 @@
       <c r="KI29" s="3"/>
       <c r="KJ29" s="3"/>
     </row>
-    <row r="30" spans="1:296" ht="19">
+    <row r="30" spans="1:296" ht="19" customHeight="1">
       <c r="A30" s="3"/>
       <c r="B30" s="3">
         <v>29</v>
@@ -12451,19 +12286,19 @@
       <c r="H30" s="8">
         <v>0</v>
       </c>
-      <c r="I30" s="18" t="s">
+      <c r="I30" s="19" t="s">
         <v>241</v>
       </c>
-      <c r="J30" s="20" t="s">
+      <c r="J30" s="21" t="s">
         <v>242</v>
       </c>
-      <c r="K30" s="18" t="s">
+      <c r="K30" s="19" t="s">
         <v>243</v>
       </c>
-      <c r="L30" s="18">
+      <c r="L30" s="19">
         <v>2022</v>
       </c>
-      <c r="M30" s="18" t="s">
+      <c r="M30" s="19" t="s">
         <v>244</v>
       </c>
       <c r="N30" s="3">
@@ -12516,7 +12351,7 @@
         <v>0</v>
       </c>
       <c r="AG30" s="3">
-        <f t="shared" ref="AG30:AG43" si="1">AC30-AF30</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="AH30" s="3" t="s">
@@ -12793,7 +12628,7 @@
       <c r="KI30" s="3"/>
       <c r="KJ30" s="3"/>
     </row>
-    <row r="31" spans="1:296" ht="19">
+    <row r="31" spans="1:296" ht="19" customHeight="1">
       <c r="A31" s="3"/>
       <c r="B31" s="3">
         <v>30</v>
@@ -12816,11 +12651,11 @@
       <c r="H31" s="8">
         <v>0</v>
       </c>
-      <c r="I31" s="18"/>
+      <c r="I31" s="23"/>
       <c r="J31" s="20"/>
-      <c r="K31" s="18"/>
-      <c r="L31" s="18"/>
-      <c r="M31" s="18"/>
+      <c r="K31" s="20"/>
+      <c r="L31" s="20"/>
+      <c r="M31" s="20"/>
       <c r="N31" s="3">
         <v>2</v>
       </c>
@@ -12873,7 +12708,7 @@
         <v>0</v>
       </c>
       <c r="AG31" s="3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>24</v>
       </c>
       <c r="AH31" s="3" t="s">
@@ -13150,7 +12985,7 @@
       <c r="KI31" s="3"/>
       <c r="KJ31" s="3"/>
     </row>
-    <row r="32" spans="1:296" ht="19">
+    <row r="32" spans="1:296" ht="19" customHeight="1">
       <c r="A32" s="3"/>
       <c r="B32" s="3">
         <v>31</v>
@@ -13173,11 +13008,11 @@
       <c r="H32" s="8">
         <v>0</v>
       </c>
-      <c r="I32" s="18"/>
+      <c r="I32" s="23"/>
       <c r="J32" s="20"/>
-      <c r="K32" s="18"/>
-      <c r="L32" s="18"/>
-      <c r="M32" s="18"/>
+      <c r="K32" s="20"/>
+      <c r="L32" s="20"/>
+      <c r="M32" s="20"/>
       <c r="N32" s="3">
         <v>3</v>
       </c>
@@ -13230,7 +13065,7 @@
         <v>0</v>
       </c>
       <c r="AG32" s="3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>25</v>
       </c>
       <c r="AH32" s="3" t="s">
@@ -13507,7 +13342,7 @@
       <c r="KI32" s="3"/>
       <c r="KJ32" s="3"/>
     </row>
-    <row r="33" spans="1:296" ht="34">
+    <row r="33" spans="1:296" ht="34" customHeight="1">
       <c r="A33" s="3"/>
       <c r="B33" s="3">
         <v>32</v>
@@ -13601,7 +13436,7 @@
         <v>0</v>
       </c>
       <c r="AG33" s="3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>105</v>
       </c>
       <c r="AH33" s="3" t="s">
@@ -13970,7 +13805,7 @@
         <v>3</v>
       </c>
       <c r="AG34" s="3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>299</v>
       </c>
       <c r="AH34" s="3" t="s">
@@ -14247,7 +14082,7 @@
       <c r="KI34" s="3"/>
       <c r="KJ34" s="3"/>
     </row>
-    <row r="35" spans="1:296" ht="19">
+    <row r="35" spans="1:296" ht="19" customHeight="1">
       <c r="A35" s="3" t="s">
         <v>277</v>
       </c>
@@ -14272,10 +14107,10 @@
       <c r="H35" s="8">
         <v>0</v>
       </c>
-      <c r="I35" s="18" t="s">
+      <c r="I35" s="19" t="s">
         <v>94</v>
       </c>
-      <c r="J35" s="20" t="s">
+      <c r="J35" s="21" t="s">
         <v>95</v>
       </c>
       <c r="K35" s="1" t="s">
@@ -14335,7 +14170,7 @@
         <v>1</v>
       </c>
       <c r="AG35" s="3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>22</v>
       </c>
       <c r="AH35" s="3" t="s">
@@ -14637,9 +14472,9 @@
       <c r="H36" s="8">
         <v>0</v>
       </c>
-      <c r="I36" s="18"/>
+      <c r="I36" s="23"/>
       <c r="J36" s="20"/>
-      <c r="K36" s="18" t="s">
+      <c r="K36" s="19" t="s">
         <v>289</v>
       </c>
       <c r="L36" s="1">
@@ -14690,7 +14525,7 @@
         <v>0</v>
       </c>
       <c r="AG36" s="3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>24</v>
       </c>
       <c r="AH36" s="3"/>
@@ -14961,7 +14796,7 @@
       <c r="KI36" s="3"/>
       <c r="KJ36" s="3"/>
     </row>
-    <row r="37" spans="1:296" ht="19">
+    <row r="37" spans="1:296" ht="19" customHeight="1">
       <c r="A37" s="3" t="s">
         <v>286</v>
       </c>
@@ -14986,10 +14821,10 @@
       <c r="H37" s="8">
         <v>0</v>
       </c>
-      <c r="I37" s="18"/>
+      <c r="I37" s="23"/>
       <c r="J37" s="20"/>
-      <c r="K37" s="18"/>
-      <c r="L37" s="18">
+      <c r="K37" s="20"/>
+      <c r="L37" s="19">
         <v>2015</v>
       </c>
       <c r="M37" s="1"/>
@@ -15037,7 +14872,7 @@
         <v>0</v>
       </c>
       <c r="AG37" s="3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="AH37" s="3"/>
@@ -15308,7 +15143,7 @@
       <c r="KI37" s="3"/>
       <c r="KJ37" s="3"/>
     </row>
-    <row r="38" spans="1:296" ht="19">
+    <row r="38" spans="1:296" ht="19" customHeight="1">
       <c r="A38" s="3" t="s">
         <v>286</v>
       </c>
@@ -15333,10 +15168,10 @@
       <c r="H38" s="8">
         <v>0</v>
       </c>
-      <c r="I38" s="18"/>
+      <c r="I38" s="23"/>
       <c r="J38" s="20"/>
-      <c r="K38" s="18"/>
-      <c r="L38" s="18"/>
+      <c r="K38" s="20"/>
+      <c r="L38" s="20"/>
       <c r="M38" s="1"/>
       <c r="N38" s="3">
         <v>2</v>
@@ -15382,7 +15217,7 @@
         <v>0</v>
       </c>
       <c r="AG38" s="3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>21</v>
       </c>
       <c r="AH38" s="3"/>
@@ -15653,7 +15488,7 @@
       <c r="KI38" s="3"/>
       <c r="KJ38" s="3"/>
     </row>
-    <row r="39" spans="1:296" ht="19">
+    <row r="39" spans="1:296" ht="19" customHeight="1">
       <c r="A39" s="3" t="s">
         <v>295</v>
       </c>
@@ -15678,15 +15513,15 @@
       <c r="H39" s="8">
         <v>0</v>
       </c>
-      <c r="I39" s="18"/>
+      <c r="I39" s="23"/>
       <c r="J39" s="20"/>
-      <c r="K39" s="18" t="s">
+      <c r="K39" s="19" t="s">
         <v>298</v>
       </c>
-      <c r="L39" s="18">
+      <c r="L39" s="19">
         <v>2014</v>
       </c>
-      <c r="M39" s="18" t="s">
+      <c r="M39" s="19" t="s">
         <v>299</v>
       </c>
       <c r="N39" s="3">
@@ -15735,7 +15570,7 @@
         <v>0</v>
       </c>
       <c r="AG39" s="3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>24</v>
       </c>
       <c r="AH39" s="3"/>
@@ -16006,7 +15841,7 @@
       <c r="KI39" s="3"/>
       <c r="KJ39" s="3"/>
     </row>
-    <row r="40" spans="1:296" ht="19">
+    <row r="40" spans="1:296" ht="19" customHeight="1">
       <c r="A40" s="3" t="s">
         <v>304</v>
       </c>
@@ -16031,11 +15866,11 @@
       <c r="H40" s="8">
         <v>0</v>
       </c>
-      <c r="I40" s="18"/>
+      <c r="I40" s="23"/>
       <c r="J40" s="20"/>
-      <c r="K40" s="18"/>
-      <c r="L40" s="18"/>
-      <c r="M40" s="18"/>
+      <c r="K40" s="20"/>
+      <c r="L40" s="20"/>
+      <c r="M40" s="20"/>
       <c r="N40" s="3">
         <v>2</v>
       </c>
@@ -16082,7 +15917,7 @@
         <v>0</v>
       </c>
       <c r="AG40" s="3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>18</v>
       </c>
       <c r="AH40" s="3"/>
@@ -16353,7 +16188,7 @@
       <c r="KI40" s="3"/>
       <c r="KJ40" s="3"/>
     </row>
-    <row r="41" spans="1:296" ht="19">
+    <row r="41" spans="1:296" ht="19" customHeight="1">
       <c r="A41" s="3" t="s">
         <v>307</v>
       </c>
@@ -16378,11 +16213,11 @@
       <c r="H41" s="8">
         <v>0</v>
       </c>
-      <c r="I41" s="18"/>
+      <c r="I41" s="23"/>
       <c r="J41" s="20"/>
-      <c r="K41" s="18"/>
-      <c r="L41" s="18"/>
-      <c r="M41" s="18"/>
+      <c r="K41" s="20"/>
+      <c r="L41" s="20"/>
+      <c r="M41" s="20"/>
       <c r="N41" s="3">
         <v>3</v>
       </c>
@@ -16429,7 +16264,7 @@
         <v>0</v>
       </c>
       <c r="AG41" s="3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>22</v>
       </c>
       <c r="AH41" s="3"/>
@@ -16700,7 +16535,7 @@
       <c r="KI41" s="3"/>
       <c r="KJ41" s="3"/>
     </row>
-    <row r="42" spans="1:296" ht="19">
+    <row r="42" spans="1:296" ht="19" customHeight="1">
       <c r="A42" s="3" t="s">
         <v>310</v>
       </c>
@@ -16725,11 +16560,11 @@
       <c r="H42" s="8">
         <v>0</v>
       </c>
-      <c r="I42" s="18"/>
+      <c r="I42" s="23"/>
       <c r="J42" s="20"/>
-      <c r="K42" s="18"/>
-      <c r="L42" s="18"/>
-      <c r="M42" s="18"/>
+      <c r="K42" s="20"/>
+      <c r="L42" s="20"/>
+      <c r="M42" s="20"/>
       <c r="N42" s="3">
         <v>4</v>
       </c>
@@ -16776,7 +16611,7 @@
         <v>0</v>
       </c>
       <c r="AG42" s="3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="AH42" s="3"/>
@@ -17047,7 +16882,7 @@
       <c r="KI42" s="3"/>
       <c r="KJ42" s="3"/>
     </row>
-    <row r="43" spans="1:296" ht="19">
+    <row r="43" spans="1:296" ht="19" customHeight="1">
       <c r="A43" s="3"/>
       <c r="B43" s="3">
         <v>42</v>
@@ -17135,7 +16970,7 @@
         <v>3</v>
       </c>
       <c r="AG43" s="3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>37</v>
       </c>
       <c r="AH43" s="3" t="s">
@@ -17412,7 +17247,7 @@
       <c r="KI43" s="3"/>
       <c r="KJ43" s="3"/>
     </row>
-    <row r="44" spans="1:296" ht="19">
+    <row r="44" spans="1:296" ht="19" customHeight="1">
       <c r="A44" s="3"/>
       <c r="B44" s="3">
         <v>43</v>
@@ -17502,7 +17337,7 @@
         <v>2</v>
       </c>
       <c r="AG44" s="3">
-        <f t="shared" ref="AG44:AG47" si="2">AC44-AF44</f>
+        <f t="shared" si="0"/>
         <v>142</v>
       </c>
       <c r="AH44" s="3" t="s">
@@ -17779,7 +17614,7 @@
       <c r="KI44" s="3"/>
       <c r="KJ44" s="3"/>
     </row>
-    <row r="45" spans="1:296" ht="68">
+    <row r="45" spans="1:296" ht="68" customHeight="1">
       <c r="A45" s="3"/>
       <c r="B45" s="3">
         <v>44</v>
@@ -17802,19 +17637,19 @@
       <c r="H45" s="7">
         <v>1</v>
       </c>
-      <c r="I45" s="18" t="s">
+      <c r="I45" s="19" t="s">
         <v>334</v>
       </c>
-      <c r="J45" s="20" t="s">
+      <c r="J45" s="21" t="s">
         <v>335</v>
       </c>
-      <c r="K45" s="18" t="s">
+      <c r="K45" s="19" t="s">
         <v>336</v>
       </c>
-      <c r="L45" s="18">
-        <v>2021</v>
-      </c>
-      <c r="M45" s="18" t="s">
+      <c r="L45" s="19">
+        <v>2022</v>
+      </c>
+      <c r="M45" s="19" t="s">
         <v>111</v>
       </c>
       <c r="N45" s="3">
@@ -17875,7 +17710,7 @@
         <v>1</v>
       </c>
       <c r="AG45" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>108</v>
       </c>
       <c r="AH45" s="3" t="s">
@@ -18152,7 +17987,7 @@
       <c r="KI45" s="3"/>
       <c r="KJ45" s="3"/>
     </row>
-    <row r="46" spans="1:296" ht="68">
+    <row r="46" spans="1:296" ht="68" customHeight="1">
       <c r="A46" s="3"/>
       <c r="B46" s="3">
         <v>45</v>
@@ -18175,11 +18010,11 @@
       <c r="H46" s="7">
         <v>1</v>
       </c>
-      <c r="I46" s="18"/>
+      <c r="I46" s="23"/>
       <c r="J46" s="20"/>
-      <c r="K46" s="18"/>
-      <c r="L46" s="18"/>
-      <c r="M46" s="18"/>
+      <c r="K46" s="20"/>
+      <c r="L46" s="20"/>
+      <c r="M46" s="20"/>
       <c r="N46" s="3">
         <v>1</v>
       </c>
@@ -18238,7 +18073,7 @@
         <v>1</v>
       </c>
       <c r="AG46" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>108</v>
       </c>
       <c r="AH46" s="3" t="s">
@@ -18515,7 +18350,7 @@
       <c r="KI46" s="3"/>
       <c r="KJ46" s="3"/>
     </row>
-    <row r="47" spans="1:296" ht="68">
+    <row r="47" spans="1:296" ht="68" customHeight="1">
       <c r="A47" s="3"/>
       <c r="B47" s="3">
         <v>46</v>
@@ -18538,11 +18373,11 @@
       <c r="H47" s="7">
         <v>1</v>
       </c>
-      <c r="I47" s="18"/>
+      <c r="I47" s="23"/>
       <c r="J47" s="20"/>
-      <c r="K47" s="18"/>
-      <c r="L47" s="18"/>
-      <c r="M47" s="18"/>
+      <c r="K47" s="20"/>
+      <c r="L47" s="20"/>
+      <c r="M47" s="20"/>
       <c r="N47" s="3">
         <v>1</v>
       </c>
@@ -18601,7 +18436,7 @@
         <v>1</v>
       </c>
       <c r="AG47" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="0"/>
         <v>108</v>
       </c>
       <c r="AH47" s="3" t="s">
@@ -18878,7 +18713,7 @@
       <c r="KI47" s="3"/>
       <c r="KJ47" s="3"/>
     </row>
-    <row r="48" spans="1:296" ht="19">
+    <row r="48" spans="1:296" ht="19" customHeight="1">
       <c r="A48" s="3"/>
       <c r="B48" s="3">
         <v>47</v>
@@ -18901,19 +18736,19 @@
       <c r="H48" s="14">
         <v>0</v>
       </c>
-      <c r="I48" s="18" t="s">
+      <c r="I48" s="19" t="s">
         <v>347</v>
       </c>
-      <c r="J48" s="20" t="s">
+      <c r="J48" s="21" t="s">
         <v>348</v>
       </c>
-      <c r="K48" s="18" t="s">
+      <c r="K48" s="19" t="s">
         <v>349</v>
       </c>
-      <c r="L48" s="18">
+      <c r="L48" s="19">
         <v>2022</v>
       </c>
-      <c r="M48" s="18" t="s">
+      <c r="M48" s="19" t="s">
         <v>350</v>
       </c>
       <c r="N48" s="3">
@@ -18970,7 +18805,7 @@
         <v>3</v>
       </c>
       <c r="AG48" s="3">
-        <f t="shared" ref="AG48:AG54" si="3">AC48-AF48</f>
+        <f t="shared" si="0"/>
         <v>27</v>
       </c>
       <c r="AH48" s="3" t="s">
@@ -19247,7 +19082,7 @@
       <c r="KI48" s="3"/>
       <c r="KJ48" s="3"/>
     </row>
-    <row r="49" spans="1:296" ht="19">
+    <row r="49" spans="1:296" ht="19" customHeight="1">
       <c r="A49" s="3"/>
       <c r="B49" s="3">
         <v>48</v>
@@ -19270,11 +19105,11 @@
       <c r="H49" s="14">
         <v>0</v>
       </c>
-      <c r="I49" s="18"/>
+      <c r="I49" s="23"/>
       <c r="J49" s="20"/>
-      <c r="K49" s="18"/>
-      <c r="L49" s="18"/>
-      <c r="M49" s="18"/>
+      <c r="K49" s="20"/>
+      <c r="L49" s="20"/>
+      <c r="M49" s="20"/>
       <c r="N49" s="3">
         <v>2</v>
       </c>
@@ -19329,7 +19164,7 @@
         <v>2</v>
       </c>
       <c r="AG49" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="0"/>
         <v>102</v>
       </c>
       <c r="AH49" s="3" t="s">
@@ -19606,7 +19441,7 @@
       <c r="KI49" s="3"/>
       <c r="KJ49" s="3"/>
     </row>
-    <row r="50" spans="1:296" ht="19">
+    <row r="50" spans="1:296" ht="19" customHeight="1">
       <c r="A50" s="3" t="s">
         <v>361</v>
       </c>
@@ -19698,7 +19533,7 @@
         <v>40</v>
       </c>
       <c r="AG50" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="0"/>
         <v>288</v>
       </c>
       <c r="AH50" s="3" t="s">
@@ -19975,7 +19810,7 @@
       <c r="KI50" s="3"/>
       <c r="KJ50" s="3"/>
     </row>
-    <row r="51" spans="1:296" ht="19">
+    <row r="51" spans="1:296" ht="19" customHeight="1">
       <c r="A51" s="3"/>
       <c r="B51" s="3">
         <v>50</v>
@@ -19998,19 +19833,19 @@
       <c r="H51" s="14">
         <v>0</v>
       </c>
-      <c r="I51" s="18" t="s">
+      <c r="I51" s="19" t="s">
         <v>181</v>
       </c>
-      <c r="J51" s="20" t="s">
+      <c r="J51" s="21" t="s">
         <v>373</v>
       </c>
-      <c r="K51" s="18" t="s">
+      <c r="K51" s="19" t="s">
         <v>183</v>
       </c>
-      <c r="L51" s="18">
+      <c r="L51" s="19">
         <v>2020</v>
       </c>
-      <c r="M51" s="18" t="s">
+      <c r="M51" s="19" t="s">
         <v>244</v>
       </c>
       <c r="N51" s="3">
@@ -20063,7 +19898,7 @@
         <v>5</v>
       </c>
       <c r="AG51" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="0"/>
         <v>18</v>
       </c>
       <c r="AH51" s="3" t="s">
@@ -20340,7 +20175,7 @@
       <c r="KI51" s="3"/>
       <c r="KJ51" s="3"/>
     </row>
-    <row r="52" spans="1:296" ht="19">
+    <row r="52" spans="1:296" ht="19" customHeight="1">
       <c r="A52" s="3"/>
       <c r="B52" s="3">
         <v>51</v>
@@ -20363,11 +20198,11 @@
       <c r="H52" s="14">
         <v>0</v>
       </c>
-      <c r="I52" s="18"/>
+      <c r="I52" s="23"/>
       <c r="J52" s="20"/>
-      <c r="K52" s="18"/>
-      <c r="L52" s="18"/>
-      <c r="M52" s="18"/>
+      <c r="K52" s="20"/>
+      <c r="L52" s="20"/>
+      <c r="M52" s="20"/>
       <c r="N52" s="3">
         <v>1</v>
       </c>
@@ -20418,7 +20253,7 @@
         <v>3</v>
       </c>
       <c r="AG52" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="0"/>
         <v>18</v>
       </c>
       <c r="AH52" s="3" t="s">
@@ -20695,7 +20530,7 @@
       <c r="KI52" s="3"/>
       <c r="KJ52" s="3"/>
     </row>
-    <row r="53" spans="1:296" ht="19">
+    <row r="53" spans="1:296" ht="19" customHeight="1">
       <c r="A53" s="3"/>
       <c r="B53" s="3">
         <v>52</v>
@@ -20718,11 +20553,11 @@
       <c r="H53" s="14">
         <v>0</v>
       </c>
-      <c r="I53" s="18"/>
+      <c r="I53" s="23"/>
       <c r="J53" s="20"/>
-      <c r="K53" s="18"/>
-      <c r="L53" s="18"/>
-      <c r="M53" s="18"/>
+      <c r="K53" s="20"/>
+      <c r="L53" s="20"/>
+      <c r="M53" s="20"/>
       <c r="N53" s="3">
         <v>1</v>
       </c>
@@ -20773,7 +20608,7 @@
         <v>0</v>
       </c>
       <c r="AG53" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="0"/>
         <v>18</v>
       </c>
       <c r="AH53" s="3" t="s">
@@ -21050,7 +20885,7 @@
       <c r="KI53" s="3"/>
       <c r="KJ53" s="3"/>
     </row>
-    <row r="54" spans="1:296" ht="19">
+    <row r="54" spans="1:296" ht="19" customHeight="1">
       <c r="A54" s="3"/>
       <c r="B54" s="3">
         <v>53</v>
@@ -21140,7 +20975,7 @@
         <v>32</v>
       </c>
       <c r="AG54" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="0"/>
         <v>348</v>
       </c>
       <c r="AH54" s="3" t="s">
@@ -21417,7 +21252,7 @@
       <c r="KI54" s="3"/>
       <c r="KJ54" s="3"/>
     </row>
-    <row r="55" spans="1:296" ht="34">
+    <row r="55" spans="1:296" ht="34" customHeight="1">
       <c r="A55" s="3"/>
       <c r="B55" s="3">
         <v>54</v>
@@ -21783,7 +21618,7 @@
       <c r="KI55" s="3"/>
       <c r="KJ55" s="3"/>
     </row>
-    <row r="56" spans="1:296" ht="19">
+    <row r="56" spans="1:296" ht="19" customHeight="1">
       <c r="A56" s="3"/>
       <c r="B56" s="3">
         <v>55</v>
@@ -21818,7 +21653,7 @@
       <c r="L56" s="1">
         <v>2023</v>
       </c>
-      <c r="M56" s="18" t="s">
+      <c r="M56" s="19" t="s">
         <v>402</v>
       </c>
       <c r="N56" s="3">
@@ -22149,7 +21984,7 @@
       <c r="KI56" s="3"/>
       <c r="KJ56" s="3"/>
     </row>
-    <row r="57" spans="1:296" ht="19">
+    <row r="57" spans="1:296" ht="19" customHeight="1">
       <c r="A57" s="3"/>
       <c r="B57" s="3">
         <v>56</v>
@@ -22184,7 +22019,7 @@
       <c r="L57" s="1">
         <v>2024</v>
       </c>
-      <c r="M57" s="18"/>
+      <c r="M57" s="20"/>
       <c r="N57" s="3">
         <v>1</v>
       </c>
@@ -22511,7 +22346,7 @@
       <c r="KI57" s="3"/>
       <c r="KJ57" s="3"/>
     </row>
-    <row r="58" spans="1:296" ht="34">
+    <row r="58" spans="1:296" ht="34" customHeight="1">
       <c r="A58" s="3"/>
       <c r="B58" s="3">
         <v>57</v>
@@ -22877,7 +22712,7 @@
       <c r="KI58" s="3"/>
       <c r="KJ58" s="3"/>
     </row>
-    <row r="59" spans="1:296" ht="19">
+    <row r="59" spans="1:296" ht="19" customHeight="1">
       <c r="A59" s="3"/>
       <c r="B59" s="3">
         <v>58</v>
@@ -23223,7 +23058,7 @@
       <c r="KI59" s="3"/>
       <c r="KJ59" s="3"/>
     </row>
-    <row r="60" spans="1:296" ht="19">
+    <row r="60" spans="1:296" ht="19" customHeight="1">
       <c r="A60" s="3"/>
       <c r="B60" s="3">
         <v>59</v>
@@ -23246,19 +23081,19 @@
       <c r="H60" s="14">
         <v>0</v>
       </c>
-      <c r="I60" s="19" t="s">
+      <c r="I60" s="22" t="s">
         <v>439</v>
       </c>
-      <c r="J60" s="20" t="s">
+      <c r="J60" s="21" t="s">
         <v>440</v>
       </c>
-      <c r="K60" s="19" t="s">
+      <c r="K60" s="22" t="s">
         <v>441</v>
       </c>
-      <c r="L60" s="18">
+      <c r="L60" s="19">
         <v>2024</v>
       </c>
-      <c r="M60" s="18" t="s">
+      <c r="M60" s="19" t="s">
         <v>402</v>
       </c>
       <c r="N60" s="3">
@@ -23581,7 +23416,7 @@
       <c r="KI60" s="3"/>
       <c r="KJ60" s="3"/>
     </row>
-    <row r="61" spans="1:296" ht="19">
+    <row r="61" spans="1:296" ht="19" customHeight="1">
       <c r="A61" s="3"/>
       <c r="B61" s="3">
         <v>60</v>
@@ -23604,11 +23439,11 @@
       <c r="H61" s="14">
         <v>0</v>
       </c>
-      <c r="I61" s="19"/>
+      <c r="I61" s="23"/>
       <c r="J61" s="20"/>
-      <c r="K61" s="19"/>
-      <c r="L61" s="18"/>
-      <c r="M61" s="18"/>
+      <c r="K61" s="20"/>
+      <c r="L61" s="20"/>
+      <c r="M61" s="20"/>
       <c r="N61" s="3">
         <v>2</v>
       </c>
@@ -23929,7 +23764,7 @@
       <c r="KI61" s="3"/>
       <c r="KJ61" s="3"/>
     </row>
-    <row r="62" spans="1:296" ht="19">
+    <row r="62" spans="1:296" ht="19" customHeight="1">
       <c r="A62" s="3"/>
       <c r="B62" s="3">
         <v>61</v>
@@ -24281,7 +24116,7 @@
       <c r="KI62" s="3"/>
       <c r="KJ62" s="3"/>
     </row>
-    <row r="63" spans="1:296" ht="19">
+    <row r="63" spans="1:296" ht="19" customHeight="1">
       <c r="A63" s="3"/>
       <c r="B63" s="3">
         <v>62</v>
@@ -24304,19 +24139,19 @@
       <c r="H63" s="14">
         <v>0</v>
       </c>
-      <c r="I63" s="18" t="s">
+      <c r="I63" s="19" t="s">
         <v>462</v>
       </c>
-      <c r="J63" s="20" t="s">
+      <c r="J63" s="21" t="s">
         <v>463</v>
       </c>
-      <c r="K63" s="18" t="s">
+      <c r="K63" s="19" t="s">
         <v>464</v>
       </c>
-      <c r="L63" s="18">
+      <c r="L63" s="19">
         <v>2024</v>
       </c>
-      <c r="M63" s="18" t="s">
+      <c r="M63" s="19" t="s">
         <v>465</v>
       </c>
       <c r="N63" s="3">
@@ -24631,7 +24466,7 @@
       <c r="KI63" s="3"/>
       <c r="KJ63" s="3"/>
     </row>
-    <row r="64" spans="1:296" ht="19">
+    <row r="64" spans="1:296" ht="19" customHeight="1">
       <c r="A64" s="3"/>
       <c r="B64" s="3">
         <v>63</v>
@@ -24654,11 +24489,11 @@
       <c r="H64" s="14">
         <v>0</v>
       </c>
-      <c r="I64" s="18"/>
+      <c r="I64" s="23"/>
       <c r="J64" s="20"/>
-      <c r="K64" s="18"/>
-      <c r="L64" s="18"/>
-      <c r="M64" s="18"/>
+      <c r="K64" s="20"/>
+      <c r="L64" s="20"/>
+      <c r="M64" s="20"/>
       <c r="N64" s="3">
         <v>1</v>
       </c>
@@ -24971,7 +24806,7 @@
       <c r="KI64" s="3"/>
       <c r="KJ64" s="3"/>
     </row>
-    <row r="65" spans="1:296" ht="16">
+    <row r="65" spans="1:296" ht="16" customHeight="1">
       <c r="A65" s="3"/>
       <c r="B65" s="3">
         <v>64</v>
@@ -24992,19 +24827,19 @@
       <c r="H65" s="14">
         <v>0</v>
       </c>
-      <c r="I65" s="18" t="s">
+      <c r="I65" s="19" t="s">
         <v>475</v>
       </c>
-      <c r="J65" s="20" t="s">
+      <c r="J65" s="21" t="s">
         <v>476</v>
       </c>
-      <c r="K65" s="18" t="s">
+      <c r="K65" s="19" t="s">
         <v>477</v>
       </c>
-      <c r="L65" s="18">
+      <c r="L65" s="19">
         <v>2023</v>
       </c>
-      <c r="M65" s="18" t="s">
+      <c r="M65" s="19" t="s">
         <v>478</v>
       </c>
       <c r="N65" s="3"/>
@@ -25315,7 +25150,7 @@
       <c r="KI65" s="3"/>
       <c r="KJ65" s="3"/>
     </row>
-    <row r="66" spans="1:296" ht="16">
+    <row r="66" spans="1:296" ht="16" customHeight="1">
       <c r="A66" s="3"/>
       <c r="B66" s="3">
         <v>65</v>
@@ -25336,11 +25171,11 @@
       <c r="H66" s="14">
         <v>0</v>
       </c>
-      <c r="I66" s="18"/>
+      <c r="I66" s="23"/>
       <c r="J66" s="20"/>
-      <c r="K66" s="18"/>
-      <c r="L66" s="18"/>
-      <c r="M66" s="18"/>
+      <c r="K66" s="20"/>
+      <c r="L66" s="20"/>
+      <c r="M66" s="20"/>
       <c r="N66" s="3"/>
       <c r="O66" s="3"/>
       <c r="P66" s="3"/>
@@ -25649,7 +25484,7 @@
       <c r="KI66" s="3"/>
       <c r="KJ66" s="3"/>
     </row>
-    <row r="67" spans="1:296" ht="16">
+    <row r="67" spans="1:296" ht="16" customHeight="1">
       <c r="A67" s="3" t="s">
         <v>484</v>
       </c>
@@ -25973,7 +25808,7 @@
       <c r="KI67" s="3"/>
       <c r="KJ67" s="3"/>
     </row>
-    <row r="68" spans="1:296" ht="16">
+    <row r="68" spans="1:296" ht="16" customHeight="1">
       <c r="A68" s="3" t="s">
         <v>374</v>
       </c>
@@ -25999,8 +25834,12 @@
       <c r="I68" s="3"/>
       <c r="J68" s="9"/>
       <c r="K68" s="1"/>
-      <c r="L68" s="1"/>
-      <c r="M68" s="1"/>
+      <c r="L68" s="1">
+        <v>2020</v>
+      </c>
+      <c r="M68" s="24" t="s">
+        <v>184</v>
+      </c>
       <c r="N68" s="3"/>
       <c r="O68" s="3"/>
       <c r="P68" s="3"/>
@@ -26029,7 +25868,7 @@
         <v>491</v>
       </c>
       <c r="AK68" s="10" t="s">
-        <v>492</v>
+        <v>515</v>
       </c>
       <c r="AL68" s="3" t="s">
         <v>90</v>
@@ -26293,16 +26132,16 @@
       <c r="KI68" s="3"/>
       <c r="KJ68" s="3"/>
     </row>
-    <row r="69" spans="1:296" ht="16">
+    <row r="69" spans="1:296" ht="16" customHeight="1">
       <c r="A69" s="3"/>
       <c r="B69" s="3">
         <v>68</v>
       </c>
       <c r="C69" s="3" t="s">
+        <v>492</v>
+      </c>
+      <c r="D69" s="3" t="s">
         <v>493</v>
-      </c>
-      <c r="D69" s="3" t="s">
-        <v>494</v>
       </c>
       <c r="E69" s="3"/>
       <c r="F69" s="7">
@@ -26338,7 +26177,7 @@
         <v>52</v>
       </c>
       <c r="AJ69" s="3" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="AK69" s="10"/>
       <c r="AL69" s="3"/>
@@ -26601,16 +26440,16 @@
       <c r="KI69" s="3"/>
       <c r="KJ69" s="3"/>
     </row>
-    <row r="70" spans="1:296" ht="16">
+    <row r="70" spans="1:296" ht="16" customHeight="1">
       <c r="A70" s="3"/>
       <c r="B70" s="3">
         <v>69</v>
       </c>
       <c r="C70" s="3" t="s">
+        <v>495</v>
+      </c>
+      <c r="D70" s="3" t="s">
         <v>496</v>
-      </c>
-      <c r="D70" s="3" t="s">
-        <v>497</v>
       </c>
       <c r="E70" s="3"/>
       <c r="F70" s="7">
@@ -26626,7 +26465,7 @@
         <v>227</v>
       </c>
       <c r="J70" s="9" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="K70" s="1"/>
       <c r="L70" s="1"/>
@@ -26668,16 +26507,16 @@
         <v>28</v>
       </c>
       <c r="AH70" s="3" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="AI70" s="3" t="s">
         <v>52</v>
       </c>
       <c r="AJ70" s="3" t="s">
+        <v>499</v>
+      </c>
+      <c r="AK70" s="10" t="s">
         <v>500</v>
-      </c>
-      <c r="AK70" s="10" t="s">
-        <v>501</v>
       </c>
       <c r="AL70" s="3" t="s">
         <v>55</v>
@@ -26941,16 +26780,16 @@
       <c r="KI70" s="3"/>
       <c r="KJ70" s="3"/>
     </row>
-    <row r="71" spans="1:296" ht="16">
+    <row r="71" spans="1:296" ht="16" customHeight="1">
       <c r="A71" s="3"/>
       <c r="B71" s="3">
         <v>70</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="D71" s="3" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="E71" s="3"/>
       <c r="F71" s="7">
@@ -26966,7 +26805,7 @@
         <v>227</v>
       </c>
       <c r="J71" s="9" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="K71" s="1"/>
       <c r="L71" s="1"/>
@@ -27008,16 +26847,16 @@
         <v>31</v>
       </c>
       <c r="AH71" s="3" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="AI71" s="3" t="s">
         <v>52</v>
       </c>
       <c r="AJ71" s="3" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="AK71" s="10" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="AL71" s="3" t="s">
         <v>55</v>
@@ -27281,16 +27120,16 @@
       <c r="KI71" s="3"/>
       <c r="KJ71" s="3"/>
     </row>
-    <row r="72" spans="1:296" ht="16">
+    <row r="72" spans="1:296" ht="16" customHeight="1">
       <c r="A72" s="3"/>
       <c r="B72" s="3">
         <v>71</v>
       </c>
       <c r="C72" s="3" t="s">
+        <v>504</v>
+      </c>
+      <c r="D72" s="3" t="s">
         <v>505</v>
-      </c>
-      <c r="D72" s="3" t="s">
-        <v>506</v>
       </c>
       <c r="E72" s="3"/>
       <c r="F72" s="7">
@@ -27346,10 +27185,10 @@
       <c r="AH72" s="3"/>
       <c r="AI72" s="3"/>
       <c r="AJ72" s="3" t="s">
+        <v>506</v>
+      </c>
+      <c r="AK72" s="10" t="s">
         <v>507</v>
-      </c>
-      <c r="AK72" s="10" t="s">
-        <v>508</v>
       </c>
       <c r="AL72" s="3" t="s">
         <v>55</v>
@@ -27613,7 +27452,7 @@
       <c r="KI72" s="3"/>
       <c r="KJ72" s="3"/>
     </row>
-    <row r="73" spans="1:296" ht="16">
+    <row r="73" spans="1:296" ht="16" customHeight="1">
       <c r="A73" s="3"/>
       <c r="B73" s="3"/>
       <c r="C73" s="3"/>
@@ -27650,10 +27489,10 @@
       <c r="AH73" s="3"/>
       <c r="AI73" s="3"/>
       <c r="AJ73" s="3" t="s">
+        <v>508</v>
+      </c>
+      <c r="AK73" s="17" t="s">
         <v>509</v>
-      </c>
-      <c r="AK73" s="17" t="s">
-        <v>510</v>
       </c>
       <c r="AL73" s="3" t="s">
         <v>90</v>
@@ -27917,7 +27756,7 @@
       <c r="KI73" s="3"/>
       <c r="KJ73" s="3"/>
     </row>
-    <row r="74" spans="1:296" ht="16">
+    <row r="74" spans="1:296" ht="16" customHeight="1">
       <c r="A74" s="3"/>
       <c r="B74" s="3"/>
       <c r="C74" s="3"/>
@@ -27956,10 +27795,10 @@
         <v>52</v>
       </c>
       <c r="AJ74" s="3" t="s">
+        <v>510</v>
+      </c>
+      <c r="AK74" s="10" t="s">
         <v>511</v>
-      </c>
-      <c r="AK74" s="10" t="s">
-        <v>512</v>
       </c>
       <c r="AL74" s="3" t="s">
         <v>90</v>
@@ -28223,7 +28062,7 @@
       <c r="KI74" s="3"/>
       <c r="KJ74" s="3"/>
     </row>
-    <row r="75" spans="1:296" ht="16">
+    <row r="75" spans="1:296" ht="16" customHeight="1">
       <c r="A75" s="3"/>
       <c r="B75" s="3"/>
       <c r="C75" s="3"/>
@@ -28521,7 +28360,7 @@
       <c r="KI75" s="3"/>
       <c r="KJ75" s="3"/>
     </row>
-    <row r="76" spans="1:296" ht="16">
+    <row r="76" spans="1:296" ht="16" customHeight="1">
       <c r="A76" s="3"/>
       <c r="B76" s="3"/>
       <c r="C76" s="3"/>
@@ -28539,185 +28378,184 @@
       <c r="R76" s="3"/>
       <c r="AK76" s="10"/>
     </row>
-    <row r="77" spans="1:296" ht="16">
+    <row r="77" spans="1:296" ht="16" customHeight="1">
       <c r="M77" s="1"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:AL74" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="88">
-    <mergeCell ref="M51:M53"/>
-    <mergeCell ref="M56:M57"/>
+    <mergeCell ref="I2:I5"/>
+    <mergeCell ref="L37:L38"/>
+    <mergeCell ref="J51:J53"/>
+    <mergeCell ref="I12:I13"/>
+    <mergeCell ref="K12:K13"/>
+    <mergeCell ref="I21:I22"/>
+    <mergeCell ref="K16:K18"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="K2:K5"/>
+    <mergeCell ref="I27:I29"/>
+    <mergeCell ref="L39:L42"/>
+    <mergeCell ref="I14:I15"/>
+    <mergeCell ref="K14:K15"/>
+    <mergeCell ref="K36:K38"/>
+    <mergeCell ref="I45:I47"/>
+    <mergeCell ref="I30:I32"/>
+    <mergeCell ref="I16:I18"/>
+    <mergeCell ref="J45:J47"/>
+    <mergeCell ref="L45:L47"/>
+    <mergeCell ref="K21:K22"/>
+    <mergeCell ref="K60:K61"/>
+    <mergeCell ref="I51:I53"/>
+    <mergeCell ref="K30:K32"/>
+    <mergeCell ref="K45:K47"/>
+    <mergeCell ref="L23:L26"/>
+    <mergeCell ref="L16:L18"/>
+    <mergeCell ref="K39:K42"/>
+    <mergeCell ref="I35:I42"/>
+    <mergeCell ref="L51:L53"/>
+    <mergeCell ref="J27:J29"/>
+    <mergeCell ref="J19:J20"/>
+    <mergeCell ref="L19:L20"/>
+    <mergeCell ref="I23:I26"/>
+    <mergeCell ref="K23:K26"/>
+    <mergeCell ref="I63:I64"/>
+    <mergeCell ref="I65:I66"/>
+    <mergeCell ref="K65:K66"/>
+    <mergeCell ref="J63:J64"/>
+    <mergeCell ref="J65:J66"/>
+    <mergeCell ref="M12:M13"/>
+    <mergeCell ref="L27:L29"/>
+    <mergeCell ref="L60:L61"/>
+    <mergeCell ref="M14:M15"/>
     <mergeCell ref="M60:M61"/>
-    <mergeCell ref="M63:M64"/>
-    <mergeCell ref="M65:M66"/>
-    <mergeCell ref="L60:L61"/>
     <mergeCell ref="L63:L64"/>
     <mergeCell ref="L65:L66"/>
-    <mergeCell ref="M2:M5"/>
-    <mergeCell ref="M7:M8"/>
-    <mergeCell ref="M12:M13"/>
-    <mergeCell ref="M14:M15"/>
-    <mergeCell ref="M16:M18"/>
+    <mergeCell ref="M56:M57"/>
     <mergeCell ref="M19:M20"/>
-    <mergeCell ref="M21:M22"/>
-    <mergeCell ref="M23:M26"/>
-    <mergeCell ref="M27:M29"/>
+    <mergeCell ref="J23:J26"/>
+    <mergeCell ref="L48:L49"/>
     <mergeCell ref="M30:M32"/>
     <mergeCell ref="M39:M42"/>
+    <mergeCell ref="M2:M5"/>
+    <mergeCell ref="K7:K8"/>
+    <mergeCell ref="J2:J5"/>
+    <mergeCell ref="L2:L5"/>
+    <mergeCell ref="I60:I61"/>
     <mergeCell ref="M45:M47"/>
+    <mergeCell ref="J16:J18"/>
+    <mergeCell ref="I7:I8"/>
+    <mergeCell ref="M65:M66"/>
+    <mergeCell ref="I48:I49"/>
+    <mergeCell ref="K48:K49"/>
+    <mergeCell ref="M21:M22"/>
+    <mergeCell ref="K51:K53"/>
+    <mergeCell ref="J12:J13"/>
+    <mergeCell ref="M51:M53"/>
+    <mergeCell ref="J21:J22"/>
+    <mergeCell ref="L21:L22"/>
+    <mergeCell ref="I19:I20"/>
+    <mergeCell ref="K19:K20"/>
+    <mergeCell ref="M63:M64"/>
     <mergeCell ref="M48:M49"/>
-    <mergeCell ref="L37:L38"/>
-    <mergeCell ref="L39:L42"/>
-    <mergeCell ref="L45:L47"/>
-    <mergeCell ref="L48:L49"/>
-    <mergeCell ref="L51:L53"/>
-    <mergeCell ref="L19:L20"/>
-    <mergeCell ref="L21:L22"/>
-    <mergeCell ref="L23:L26"/>
-    <mergeCell ref="L27:L29"/>
+    <mergeCell ref="J60:J61"/>
+    <mergeCell ref="K63:K64"/>
+    <mergeCell ref="L12:L13"/>
+    <mergeCell ref="M7:M8"/>
+    <mergeCell ref="L14:L15"/>
+    <mergeCell ref="J35:J42"/>
+    <mergeCell ref="J14:J15"/>
+    <mergeCell ref="J30:J32"/>
     <mergeCell ref="L30:L32"/>
-    <mergeCell ref="L2:L5"/>
+    <mergeCell ref="M16:M18"/>
+    <mergeCell ref="M23:M26"/>
     <mergeCell ref="L7:L8"/>
-    <mergeCell ref="L12:L13"/>
-    <mergeCell ref="L14:L15"/>
-    <mergeCell ref="L16:L18"/>
-    <mergeCell ref="K48:K49"/>
-    <mergeCell ref="K51:K53"/>
-    <mergeCell ref="K60:K61"/>
-    <mergeCell ref="K63:K64"/>
-    <mergeCell ref="K65:K66"/>
-    <mergeCell ref="J60:J61"/>
-    <mergeCell ref="J63:J64"/>
-    <mergeCell ref="J65:J66"/>
-    <mergeCell ref="K2:K5"/>
-    <mergeCell ref="K7:K8"/>
-    <mergeCell ref="K12:K13"/>
-    <mergeCell ref="K14:K15"/>
-    <mergeCell ref="K16:K18"/>
-    <mergeCell ref="K19:K20"/>
-    <mergeCell ref="K21:K22"/>
-    <mergeCell ref="K23:K26"/>
     <mergeCell ref="K27:K29"/>
-    <mergeCell ref="K30:K32"/>
-    <mergeCell ref="K36:K38"/>
-    <mergeCell ref="K39:K42"/>
-    <mergeCell ref="K45:K47"/>
-    <mergeCell ref="I63:I64"/>
-    <mergeCell ref="I65:I66"/>
-    <mergeCell ref="J2:J5"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="J12:J13"/>
-    <mergeCell ref="J14:J15"/>
-    <mergeCell ref="J16:J18"/>
-    <mergeCell ref="J19:J20"/>
-    <mergeCell ref="J21:J22"/>
-    <mergeCell ref="J23:J26"/>
-    <mergeCell ref="J27:J29"/>
-    <mergeCell ref="J30:J32"/>
-    <mergeCell ref="J35:J42"/>
-    <mergeCell ref="J45:J47"/>
     <mergeCell ref="J48:J49"/>
-    <mergeCell ref="J51:J53"/>
-    <mergeCell ref="I35:I42"/>
-    <mergeCell ref="I45:I47"/>
-    <mergeCell ref="I48:I49"/>
-    <mergeCell ref="I51:I53"/>
-    <mergeCell ref="I60:I61"/>
-    <mergeCell ref="I19:I20"/>
-    <mergeCell ref="I21:I22"/>
-    <mergeCell ref="I23:I26"/>
-    <mergeCell ref="I27:I29"/>
-    <mergeCell ref="I30:I32"/>
-    <mergeCell ref="I2:I5"/>
-    <mergeCell ref="I7:I8"/>
-    <mergeCell ref="I12:I13"/>
-    <mergeCell ref="I14:I15"/>
-    <mergeCell ref="I16:I18"/>
+    <mergeCell ref="M27:M29"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="M58" r:id="rId1" tooltip="https://link.springer.com/journal/13415" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="J2" r:id="rId2" tooltip="mailto:merryndconstable@gmail.com" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="J6" r:id="rId3" tooltip="mailto:merryndconstable@gmail.com" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="J9" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="J12" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="J14" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="J16" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="J19" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="J11" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="J21" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="J23" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="J27" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="J35" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="J54" r:id="rId14" tooltip="mailto:wf3126@mail.tsinghua.edu.cn" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="J56" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
-    <hyperlink ref="J57" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="AK21" r:id="rId17" tooltip="https://osf.io/8bktn/" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="AK22" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="AK2" r:id="rId19" tooltip="https://osf.io/sejw7/" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="AK3" r:id="rId20" tooltip="https://osf.io/sejw7/" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
-    <hyperlink ref="AK4" r:id="rId21" tooltip="https://osf.io/sejw7/" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
-    <hyperlink ref="AK5" r:id="rId22" tooltip="https://osf.io/sejw7/" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
-    <hyperlink ref="AK6" r:id="rId23" tooltip="https://osf.io/5zaej/" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
-    <hyperlink ref="AK9" r:id="rId24" tooltip="https://osf.io/4zvkm/" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
-    <hyperlink ref="AK12" r:id="rId25" tooltip="https://osf.io/khyjq/" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
-    <hyperlink ref="AK23" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
-    <hyperlink ref="AK24" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
-    <hyperlink ref="AK25" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
-    <hyperlink ref="AK26" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
-    <hyperlink ref="AK27" r:id="rId30" tooltip="https://osf.io/3ke4f/" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
-    <hyperlink ref="AK28" r:id="rId31" tooltip="https://osf.io/3ke4f/" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
-    <hyperlink ref="AK29" r:id="rId32" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
-    <hyperlink ref="AK43" r:id="rId33" tooltip="https://osf.io/2juxk/?view_only=b4e01124337a4801b4beb99dbe803b8d" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
-    <hyperlink ref="AK44" r:id="rId34" tooltip="https://researchdata.bath.ac.uk/924/" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
-    <hyperlink ref="AK30" r:id="rId35" tooltip="https://osf.io/cj7fp/" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
-    <hyperlink ref="AK31" r:id="rId36" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
-    <hyperlink ref="AK32" r:id="rId37" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
-    <hyperlink ref="AK34" r:id="rId38" tooltip="https://osf.io/4n6j7/" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
-    <hyperlink ref="AK35" r:id="rId39" tooltip="https://zenodo.org/records/8031086" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
-    <hyperlink ref="AK45" r:id="rId40" tooltip="https://osf.io/u9ty6/?view_only=9bdbbaf95f9a4d9c8bc53dd1a29563ae." xr:uid="{00000000-0004-0000-0000-000027000000}"/>
-    <hyperlink ref="AK48" r:id="rId41" tooltip="https://doi.org/10.17605/OSF.IO/FE3JW" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
-    <hyperlink ref="AK49" r:id="rId42" xr:uid="{00000000-0004-0000-0000-000029000000}"/>
-    <hyperlink ref="AK50" r:id="rId43" tooltip="https://doi.org/10.26180/20011142" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
-    <hyperlink ref="AK51" r:id="rId44" tooltip="https://osf.io/35wp9" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
-    <hyperlink ref="AK52" r:id="rId45" tooltip="https://osf.io/35wp9" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
-    <hyperlink ref="AK53" r:id="rId46" tooltip="https://osf.io/35wp9" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
-    <hyperlink ref="AK54" r:id="rId47" tooltip="https://osf.io/hbrus/?view_only=98b2095f72e64fd382fc0d33de3f4497" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
-    <hyperlink ref="AK20" r:id="rId48" location="sec025" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
-    <hyperlink ref="AK19" r:id="rId49" location="sec025" tooltip="https://journals.plos.org/plosone/article?id=10.1371/journal.pone.0190679#sec025" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
-    <hyperlink ref="AK57" r:id="rId50" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
-    <hyperlink ref="AK58" r:id="rId51" tooltip="https://doi.org/10.3758/s13415-024-01157-0" xr:uid="{00000000-0004-0000-0000-000032000000}"/>
-    <hyperlink ref="AK60" r:id="rId52" tooltip="https://doi.org/10.17605/OSF.IO/XA4H8" xr:uid="{00000000-0004-0000-0000-000033000000}"/>
-    <hyperlink ref="AK61" r:id="rId53" tooltip="https://doi.org/10.17605/OSF.IO/XA4H8" xr:uid="{00000000-0004-0000-0000-000034000000}"/>
-    <hyperlink ref="AK62" r:id="rId54" tooltip="https://osf.io/br98c/" xr:uid="{00000000-0004-0000-0000-000035000000}"/>
-    <hyperlink ref="J63" r:id="rId55" xr:uid="{00000000-0004-0000-0000-000036000000}"/>
-    <hyperlink ref="AK63" r:id="rId56" xr:uid="{00000000-0004-0000-0000-000037000000}"/>
-    <hyperlink ref="J59" r:id="rId57" xr:uid="{00000000-0004-0000-0000-000038000000}"/>
-    <hyperlink ref="J64" r:id="rId58" display="mailto:n.kirk@abertay.ac.uk" xr:uid="{00000000-0004-0000-0000-000039000000}"/>
-    <hyperlink ref="AK64" r:id="rId59" xr:uid="{00000000-0004-0000-0000-00003A000000}"/>
-    <hyperlink ref="AK46" r:id="rId60" tooltip="https://osf.io/u9ty6/?view_only=9bdbbaf95f9a4d9c8bc53dd1a29563ae." xr:uid="{00000000-0004-0000-0000-00003B000000}"/>
-    <hyperlink ref="AK47" r:id="rId61" tooltip="https://osf.io/u9ty6/?view_only=9bdbbaf95f9a4d9c8bc53dd1a29563ae." xr:uid="{00000000-0004-0000-0000-00003C000000}"/>
-    <hyperlink ref="AK65" r:id="rId62" xr:uid="{00000000-0004-0000-0000-00003D000000}"/>
-    <hyperlink ref="AK66" r:id="rId63" xr:uid="{00000000-0004-0000-0000-00003E000000}"/>
-    <hyperlink ref="AK67" r:id="rId64" xr:uid="{00000000-0004-0000-0000-00003F000000}"/>
-    <hyperlink ref="AK68" r:id="rId65" xr:uid="{00000000-0004-0000-0000-000040000000}"/>
-    <hyperlink ref="AK14" r:id="rId66" tooltip="https://osf.io/bw27c" xr:uid="{00000000-0004-0000-0000-000041000000}"/>
-    <hyperlink ref="AK15" r:id="rId67" xr:uid="{00000000-0004-0000-0000-000042000000}"/>
-    <hyperlink ref="AK7" r:id="rId68" xr:uid="{00000000-0004-0000-0000-000043000000}"/>
-    <hyperlink ref="AK8" r:id="rId69" xr:uid="{00000000-0004-0000-0000-000044000000}"/>
-    <hyperlink ref="AK70" r:id="rId70" xr:uid="{00000000-0004-0000-0000-000045000000}"/>
-    <hyperlink ref="AK71" r:id="rId71" xr:uid="{00000000-0004-0000-0000-000046000000}"/>
-    <hyperlink ref="AK72" r:id="rId72" tooltip="https://osf.io/zyauc/." xr:uid="{00000000-0004-0000-0000-000047000000}"/>
-    <hyperlink ref="AK16" r:id="rId73" tooltip="http://dx.doi.org/10.23668/psycharchives.2642" xr:uid="{00000000-0004-0000-0000-000048000000}"/>
-    <hyperlink ref="AK11" r:id="rId74" tooltip="https://figshare.com/s/e1391ebe3f11e8d70d9f" xr:uid="{00000000-0004-0000-0000-000049000000}"/>
-    <hyperlink ref="AK59" r:id="rId75" xr:uid="{00000000-0004-0000-0000-00004A000000}"/>
-    <hyperlink ref="AK73" r:id="rId76" tooltip="https://osf.io/ehu75" xr:uid="{00000000-0004-0000-0000-00004B000000}"/>
-    <hyperlink ref="AK74" r:id="rId77" xr:uid="{00000000-0004-0000-0000-00004C000000}"/>
-    <hyperlink ref="AK17" r:id="rId78" tooltip="http://dx.doi.org/10.23668/psycharchives.2642" xr:uid="{00000000-0004-0000-0000-00004D000000}"/>
-    <hyperlink ref="AK18" r:id="rId79" tooltip="http://dx.doi.org/10.23668/psycharchives.2642" xr:uid="{00000000-0004-0000-0000-00004E000000}"/>
-    <hyperlink ref="J62" r:id="rId80" xr:uid="{00000000-0004-0000-0000-00004F000000}"/>
-    <hyperlink ref="AK13" r:id="rId81" xr:uid="{00000000-0004-0000-0000-000050000000}"/>
-    <hyperlink ref="J70" r:id="rId82" xr:uid="{00000000-0004-0000-0000-000051000000}"/>
-    <hyperlink ref="J71" r:id="rId83" xr:uid="{00000000-0004-0000-0000-000052000000}"/>
+    <hyperlink ref="J2" r:id="rId1" tooltip="mailto:merryndconstable@gmail.com" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="AK2" r:id="rId2" tooltip="https://osf.io/sejw7/" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="AK3" r:id="rId3" tooltip="https://osf.io/sejw7/" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="AK4" r:id="rId4" tooltip="https://osf.io/sejw7/" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="AK5" r:id="rId5" tooltip="https://osf.io/sejw7/" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="J6" r:id="rId6" tooltip="mailto:merryndconstable@gmail.com" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="AK6" r:id="rId7" tooltip="https://osf.io/5zaej/" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="AK7" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="AK8" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="J9" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="AK9" r:id="rId11" tooltip="https://osf.io/4zvkm/" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="J11" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="AK11" r:id="rId13" tooltip="https://figshare.com/s/e1391ebe3f11e8d70d9f" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="J12" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="AK12" r:id="rId15" tooltip="https://osf.io/khyjq/" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="AK13" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="J14" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="AK14" r:id="rId18" tooltip="https://osf.io/bw27c" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="AK15" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="J16" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="AK16" r:id="rId21" tooltip="http://dx.doi.org/10.23668/psycharchives.2642" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="AK17" r:id="rId22" tooltip="http://dx.doi.org/10.23668/psycharchives.2642" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="AK18" r:id="rId23" tooltip="http://dx.doi.org/10.23668/psycharchives.2642" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="J19" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="AK19" r:id="rId25" location="sec025" tooltip="https://journals.plos.org/plosone/article?id=10.1371/journal.pone.0190679#sec025" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="AK20" r:id="rId26" location="sec025" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="J21" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
+    <hyperlink ref="AK21" r:id="rId28" tooltip="https://osf.io/8bktn/" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
+    <hyperlink ref="AK22" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
+    <hyperlink ref="J23" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
+    <hyperlink ref="AK23" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
+    <hyperlink ref="AK24" r:id="rId32" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
+    <hyperlink ref="AK25" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
+    <hyperlink ref="AK26" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
+    <hyperlink ref="J27" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
+    <hyperlink ref="AK27" r:id="rId36" tooltip="https://osf.io/3ke4f/" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
+    <hyperlink ref="AK28" r:id="rId37" tooltip="https://osf.io/3ke4f/" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
+    <hyperlink ref="AK29" r:id="rId38" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
+    <hyperlink ref="AK30" r:id="rId39" tooltip="https://osf.io/cj7fp/" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
+    <hyperlink ref="AK31" r:id="rId40" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
+    <hyperlink ref="AK32" r:id="rId41" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
+    <hyperlink ref="AK34" r:id="rId42" tooltip="https://osf.io/4n6j7/" xr:uid="{00000000-0004-0000-0000-000029000000}"/>
+    <hyperlink ref="J35" r:id="rId43" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
+    <hyperlink ref="AK35" r:id="rId44" tooltip="https://zenodo.org/records/8031086" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
+    <hyperlink ref="AK43" r:id="rId45" tooltip="https://osf.io/2juxk/?view_only=b4e01124337a4801b4beb99dbe803b8d" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
+    <hyperlink ref="AK44" r:id="rId46" tooltip="https://researchdata.bath.ac.uk/924/" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
+    <hyperlink ref="AK45" r:id="rId47" tooltip="https://osf.io/u9ty6/?view_only=9bdbbaf95f9a4d9c8bc53dd1a29563ae." xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
+    <hyperlink ref="AK46" r:id="rId48" tooltip="https://osf.io/u9ty6/?view_only=9bdbbaf95f9a4d9c8bc53dd1a29563ae." xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
+    <hyperlink ref="AK47" r:id="rId49" tooltip="https://osf.io/u9ty6/?view_only=9bdbbaf95f9a4d9c8bc53dd1a29563ae." xr:uid="{00000000-0004-0000-0000-000030000000}"/>
+    <hyperlink ref="AK48" r:id="rId50" tooltip="https://doi.org/10.17605/OSF.IO/FE3JW" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
+    <hyperlink ref="AK49" r:id="rId51" xr:uid="{00000000-0004-0000-0000-000032000000}"/>
+    <hyperlink ref="AK50" r:id="rId52" tooltip="https://doi.org/10.26180/20011142" xr:uid="{00000000-0004-0000-0000-000033000000}"/>
+    <hyperlink ref="AK51" r:id="rId53" tooltip="https://osf.io/35wp9" xr:uid="{00000000-0004-0000-0000-000034000000}"/>
+    <hyperlink ref="AK52" r:id="rId54" tooltip="https://osf.io/35wp9" xr:uid="{00000000-0004-0000-0000-000035000000}"/>
+    <hyperlink ref="AK53" r:id="rId55" tooltip="https://osf.io/35wp9" xr:uid="{00000000-0004-0000-0000-000036000000}"/>
+    <hyperlink ref="J54" r:id="rId56" tooltip="mailto:wf3126@mail.tsinghua.edu.cn" xr:uid="{00000000-0004-0000-0000-000037000000}"/>
+    <hyperlink ref="AK54" r:id="rId57" tooltip="https://osf.io/hbrus/?view_only=98b2095f72e64fd382fc0d33de3f4497" xr:uid="{00000000-0004-0000-0000-000038000000}"/>
+    <hyperlink ref="J56" r:id="rId58" xr:uid="{00000000-0004-0000-0000-000039000000}"/>
+    <hyperlink ref="J57" r:id="rId59" xr:uid="{00000000-0004-0000-0000-00003A000000}"/>
+    <hyperlink ref="AK57" r:id="rId60" xr:uid="{00000000-0004-0000-0000-00003B000000}"/>
+    <hyperlink ref="M58" r:id="rId61" tooltip="https://link.springer.com/journal/13415" xr:uid="{00000000-0004-0000-0000-00003C000000}"/>
+    <hyperlink ref="AK58" r:id="rId62" tooltip="https://doi.org/10.3758/s13415-024-01157-0" xr:uid="{00000000-0004-0000-0000-00003D000000}"/>
+    <hyperlink ref="J59" r:id="rId63" xr:uid="{00000000-0004-0000-0000-00003E000000}"/>
+    <hyperlink ref="AK59" r:id="rId64" xr:uid="{00000000-0004-0000-0000-00003F000000}"/>
+    <hyperlink ref="AK60" r:id="rId65" tooltip="https://doi.org/10.17605/OSF.IO/XA4H8" xr:uid="{00000000-0004-0000-0000-000040000000}"/>
+    <hyperlink ref="AK61" r:id="rId66" tooltip="https://doi.org/10.17605/OSF.IO/XA4H8" xr:uid="{00000000-0004-0000-0000-000041000000}"/>
+    <hyperlink ref="J62" r:id="rId67" xr:uid="{00000000-0004-0000-0000-000042000000}"/>
+    <hyperlink ref="AK62" r:id="rId68" tooltip="https://osf.io/br98c/" xr:uid="{00000000-0004-0000-0000-000043000000}"/>
+    <hyperlink ref="J63" r:id="rId69" display="mailto:n.kirk@abertay.ac.uk" xr:uid="{00000000-0004-0000-0000-000044000000}"/>
+    <hyperlink ref="AK63" r:id="rId70" xr:uid="{00000000-0004-0000-0000-000045000000}"/>
+    <hyperlink ref="AK64" r:id="rId71" xr:uid="{00000000-0004-0000-0000-000046000000}"/>
+    <hyperlink ref="AK65" r:id="rId72" xr:uid="{00000000-0004-0000-0000-000047000000}"/>
+    <hyperlink ref="AK66" r:id="rId73" xr:uid="{00000000-0004-0000-0000-000048000000}"/>
+    <hyperlink ref="AK67" r:id="rId74" xr:uid="{00000000-0004-0000-0000-000049000000}"/>
+    <hyperlink ref="AK68" r:id="rId75" xr:uid="{00000000-0004-0000-0000-00004A000000}"/>
+    <hyperlink ref="J70" r:id="rId76" xr:uid="{00000000-0004-0000-0000-00004B000000}"/>
+    <hyperlink ref="AK70" r:id="rId77" xr:uid="{00000000-0004-0000-0000-00004C000000}"/>
+    <hyperlink ref="J71" r:id="rId78" xr:uid="{00000000-0004-0000-0000-00004D000000}"/>
+    <hyperlink ref="AK71" r:id="rId79" xr:uid="{00000000-0004-0000-0000-00004E000000}"/>
+    <hyperlink ref="AK72" r:id="rId80" tooltip="https://osf.io/zyauc/." xr:uid="{00000000-0004-0000-0000-00004F000000}"/>
+    <hyperlink ref="AK73" r:id="rId81" tooltip="https://osf.io/ehu75" xr:uid="{00000000-0004-0000-0000-000050000000}"/>
+    <hyperlink ref="AK74" r:id="rId82" xr:uid="{00000000-0004-0000-0000-000051000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -28729,13 +28567,13 @@
   <dimension ref="A1:L67"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.6640625" customWidth="1"/>
-    <col min="2" max="2" width="9.1640625" customWidth="1"/>
-    <col min="3" max="3" width="6" customWidth="1"/>
-    <col min="4" max="4" width="25.6640625" customWidth="1"/>
+    <col min="1" max="1" width="3.6640625" style="18" customWidth="1"/>
+    <col min="2" max="2" width="9.1640625" style="18" customWidth="1"/>
+    <col min="3" max="3" width="6" style="18" customWidth="1"/>
+    <col min="4" max="4" width="25.6640625" style="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="16">
+    <row r="1" spans="1:12" ht="16" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -28749,7 +28587,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="16">
+    <row r="2" spans="1:12" ht="16" customHeight="1">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -28763,7 +28601,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="16">
+    <row r="3" spans="1:12" ht="16" customHeight="1">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -28777,7 +28615,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="16">
+    <row r="4" spans="1:12" ht="16" customHeight="1">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -28791,7 +28629,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="16">
+    <row r="5" spans="1:12" ht="16" customHeight="1">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -28805,7 +28643,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="16">
+    <row r="6" spans="1:12" ht="16" customHeight="1">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -28820,7 +28658,7 @@
       </c>
       <c r="L6" s="4"/>
     </row>
-    <row r="7" spans="1:12" ht="16">
+    <row r="7" spans="1:12" ht="16" customHeight="1">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -28834,7 +28672,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="16">
+    <row r="8" spans="1:12" ht="16" customHeight="1">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -28848,7 +28686,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="16">
+    <row r="9" spans="1:12" ht="16" customHeight="1">
       <c r="A9" s="3">
         <v>8</v>
       </c>
@@ -28862,7 +28700,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="16">
+    <row r="10" spans="1:12" ht="16" customHeight="1">
       <c r="A10" s="3">
         <v>9</v>
       </c>
@@ -28876,7 +28714,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="16">
+    <row r="11" spans="1:12" ht="16" customHeight="1">
       <c r="A11" s="3">
         <v>10</v>
       </c>
@@ -28890,7 +28728,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="16">
+    <row r="12" spans="1:12" ht="16" customHeight="1">
       <c r="A12" s="3">
         <v>11</v>
       </c>
@@ -28904,7 +28742,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="16">
+    <row r="13" spans="1:12" ht="16" customHeight="1">
       <c r="A13" s="3">
         <v>12</v>
       </c>
@@ -28918,7 +28756,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="16">
+    <row r="14" spans="1:12" ht="16" customHeight="1">
       <c r="A14" s="3">
         <v>13</v>
       </c>
@@ -28932,7 +28770,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="16">
+    <row r="15" spans="1:12" ht="16" customHeight="1">
       <c r="A15" s="3">
         <v>14</v>
       </c>
@@ -28946,7 +28784,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="16" spans="1:12" ht="16">
+    <row r="16" spans="1:12" ht="16" customHeight="1">
       <c r="A16" s="3">
         <v>15</v>
       </c>
@@ -28960,7 +28798,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="16">
+    <row r="17" spans="1:4" ht="16" customHeight="1">
       <c r="A17" s="3">
         <v>16</v>
       </c>
@@ -28974,7 +28812,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="16">
+    <row r="18" spans="1:4" ht="16" customHeight="1">
       <c r="A18" s="3">
         <v>17</v>
       </c>
@@ -28988,7 +28826,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="16">
+    <row r="19" spans="1:4" ht="16" customHeight="1">
       <c r="A19" s="3">
         <v>18</v>
       </c>
@@ -29002,7 +28840,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="16">
+    <row r="20" spans="1:4" ht="16" customHeight="1">
       <c r="A20" s="3">
         <v>19</v>
       </c>
@@ -29016,7 +28854,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="16">
+    <row r="21" spans="1:4" ht="16" customHeight="1">
       <c r="A21" s="3">
         <v>20</v>
       </c>
@@ -29030,7 +28868,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="16">
+    <row r="22" spans="1:4" ht="16" customHeight="1">
       <c r="A22" s="3">
         <v>21</v>
       </c>
@@ -29044,7 +28882,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="16">
+    <row r="23" spans="1:4" ht="16" customHeight="1">
       <c r="A23" s="3">
         <v>22</v>
       </c>
@@ -29058,7 +28896,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="16">
+    <row r="24" spans="1:4" ht="16" customHeight="1">
       <c r="A24" s="3">
         <v>23</v>
       </c>
@@ -29072,7 +28910,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="16">
+    <row r="25" spans="1:4" ht="16" customHeight="1">
       <c r="A25" s="3">
         <v>24</v>
       </c>
@@ -29086,7 +28924,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="26" spans="1:4" ht="16">
+    <row r="26" spans="1:4" ht="16" customHeight="1">
       <c r="A26" s="3">
         <v>25</v>
       </c>
@@ -29100,7 +28938,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="16">
+    <row r="27" spans="1:4" ht="16" customHeight="1">
       <c r="A27" s="3">
         <v>26</v>
       </c>
@@ -29114,7 +28952,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="16">
+    <row r="28" spans="1:4" ht="16" customHeight="1">
       <c r="A28" s="3">
         <v>27</v>
       </c>
@@ -29125,10 +28963,10 @@
         <v>256</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="16">
+    <row r="29" spans="1:4" ht="16" customHeight="1">
       <c r="A29" s="3">
         <v>28</v>
       </c>
@@ -29142,7 +28980,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="30" spans="1:4" ht="16">
+    <row r="30" spans="1:4" ht="16" customHeight="1">
       <c r="A30" s="3">
         <v>29</v>
       </c>
@@ -29156,7 +28994,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="31" spans="1:4" ht="16">
+    <row r="31" spans="1:4" ht="16" customHeight="1">
       <c r="A31" s="3">
         <v>30</v>
       </c>
@@ -29170,7 +29008,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="32" spans="1:4" ht="16">
+    <row r="32" spans="1:4" ht="16" customHeight="1">
       <c r="A32" s="3">
         <v>31</v>
       </c>
@@ -29184,7 +29022,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="33" spans="1:4" ht="16">
+    <row r="33" spans="1:4" ht="16" customHeight="1">
       <c r="A33" s="3">
         <v>32</v>
       </c>
@@ -29198,7 +29036,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="34" spans="1:4" ht="16">
+    <row r="34" spans="1:4" ht="16" customHeight="1">
       <c r="A34" s="3">
         <v>33</v>
       </c>
@@ -29212,7 +29050,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="35" spans="1:4" ht="16">
+    <row r="35" spans="1:4" ht="16" customHeight="1">
       <c r="A35" s="3">
         <v>34</v>
       </c>
@@ -29226,7 +29064,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="36" spans="1:4" ht="16">
+    <row r="36" spans="1:4" ht="16" customHeight="1">
       <c r="A36" s="3">
         <v>35</v>
       </c>
@@ -29240,7 +29078,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="37" spans="1:4" ht="16">
+    <row r="37" spans="1:4" ht="16" customHeight="1">
       <c r="A37" s="3">
         <v>36</v>
       </c>
@@ -29254,7 +29092,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="38" spans="1:4" ht="16">
+    <row r="38" spans="1:4" ht="16" customHeight="1">
       <c r="A38" s="3">
         <v>37</v>
       </c>
@@ -29268,7 +29106,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="39" spans="1:4" ht="16">
+    <row r="39" spans="1:4" ht="16" customHeight="1">
       <c r="A39" s="3">
         <v>38</v>
       </c>
@@ -29282,7 +29120,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="40" spans="1:4" ht="16">
+    <row r="40" spans="1:4" ht="16" customHeight="1">
       <c r="A40" s="3">
         <v>39</v>
       </c>
@@ -29293,22 +29131,22 @@
         <v>333</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>514</v>
+        <v>340</v>
       </c>
     </row>
-    <row r="41" spans="1:4" ht="16">
+    <row r="41" spans="1:4" ht="16" customHeight="1">
       <c r="A41" s="3">
         <v>40</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="D41" s="3"/>
     </row>
-    <row r="42" spans="1:4" ht="16">
+    <row r="42" spans="1:4" ht="16" customHeight="1">
       <c r="A42" s="3">
         <v>41</v>
       </c>
@@ -29322,7 +29160,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="43" spans="1:4" ht="16">
+    <row r="43" spans="1:4" ht="16" customHeight="1">
       <c r="A43" s="3">
         <v>42</v>
       </c>
@@ -29336,7 +29174,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="44" spans="1:4" ht="16">
+    <row r="44" spans="1:4" ht="16" customHeight="1">
       <c r="A44" s="3">
         <v>43</v>
       </c>
@@ -29350,7 +29188,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="45" spans="1:4" ht="16">
+    <row r="45" spans="1:4" ht="16" customHeight="1">
       <c r="A45" s="3">
         <v>44</v>
       </c>
@@ -29364,7 +29202,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="46" spans="1:4" ht="16">
+    <row r="46" spans="1:4" ht="16" customHeight="1">
       <c r="A46" s="3">
         <v>45</v>
       </c>
@@ -29378,7 +29216,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="47" spans="1:4" ht="16">
+    <row r="47" spans="1:4" ht="16" customHeight="1">
       <c r="A47" s="3">
         <v>46</v>
       </c>
@@ -29392,7 +29230,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="48" spans="1:4" ht="16">
+    <row r="48" spans="1:4" ht="16" customHeight="1">
       <c r="A48" s="3">
         <v>47</v>
       </c>
@@ -29406,7 +29244,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="49" spans="1:4" ht="16">
+    <row r="49" spans="1:4" ht="16" customHeight="1">
       <c r="A49" s="3">
         <v>48</v>
       </c>
@@ -29420,7 +29258,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="50" spans="1:4" ht="16">
+    <row r="50" spans="1:4" ht="16" customHeight="1">
       <c r="A50" s="3">
         <v>49</v>
       </c>
@@ -29434,7 +29272,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="51" spans="1:4" ht="16">
+    <row r="51" spans="1:4" ht="16" customHeight="1">
       <c r="A51" s="3">
         <v>50</v>
       </c>
@@ -29448,7 +29286,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="52" spans="1:4" ht="16">
+    <row r="52" spans="1:4" ht="16" customHeight="1">
       <c r="A52" s="3">
         <v>51</v>
       </c>
@@ -29462,7 +29300,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="53" spans="1:4" ht="16">
+    <row r="53" spans="1:4" ht="16" customHeight="1">
       <c r="A53" s="3">
         <v>52</v>
       </c>
@@ -29476,7 +29314,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="54" spans="1:4" ht="16">
+    <row r="54" spans="1:4" ht="16" customHeight="1">
       <c r="A54" s="3">
         <v>53</v>
       </c>
@@ -29490,7 +29328,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="55" spans="1:4" ht="16">
+    <row r="55" spans="1:4" ht="16" customHeight="1">
       <c r="A55" s="3">
         <v>54</v>
       </c>
@@ -29504,7 +29342,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="56" spans="1:4" ht="16">
+    <row r="56" spans="1:4" ht="16" customHeight="1">
       <c r="A56" s="3">
         <v>55</v>
       </c>
@@ -29518,7 +29356,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="57" spans="1:4" ht="16">
+    <row r="57" spans="1:4" ht="16" customHeight="1">
       <c r="A57" s="3">
         <v>56</v>
       </c>
@@ -29532,7 +29370,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="58" spans="1:4" ht="16">
+    <row r="58" spans="1:4" ht="16" customHeight="1">
       <c r="A58" s="3">
         <v>57</v>
       </c>
@@ -29546,7 +29384,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="59" spans="1:4" ht="16">
+    <row r="59" spans="1:4" ht="16" customHeight="1">
       <c r="A59" s="3">
         <v>58</v>
       </c>
@@ -29560,7 +29398,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="60" spans="1:4" ht="16">
+    <row r="60" spans="1:4" ht="16" customHeight="1">
       <c r="A60" s="3">
         <v>59</v>
       </c>
@@ -29574,7 +29412,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="61" spans="1:4" ht="16">
+    <row r="61" spans="1:4" ht="16" customHeight="1">
       <c r="A61" s="3">
         <v>60</v>
       </c>
@@ -29588,61 +29426,61 @@
         <v>491</v>
       </c>
     </row>
-    <row r="62" spans="1:4" ht="16">
+    <row r="62" spans="1:4" ht="16" customHeight="1">
       <c r="A62" s="3">
         <v>61</v>
       </c>
       <c r="B62" s="3" t="s">
+        <v>492</v>
+      </c>
+      <c r="C62" s="3" t="s">
         <v>493</v>
       </c>
-      <c r="C62" s="3" t="s">
+      <c r="D62" s="3" t="s">
         <v>494</v>
       </c>
-      <c r="D62" s="3" t="s">
-        <v>495</v>
-      </c>
     </row>
-    <row r="63" spans="1:4" ht="16">
+    <row r="63" spans="1:4" ht="16" customHeight="1">
       <c r="A63" s="3">
         <v>62</v>
       </c>
       <c r="B63" s="3" t="s">
+        <v>495</v>
+      </c>
+      <c r="C63" s="3" t="s">
         <v>496</v>
       </c>
-      <c r="C63" s="3" t="s">
-        <v>497</v>
-      </c>
       <c r="D63" s="3" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
     </row>
-    <row r="64" spans="1:4" ht="16">
+    <row r="64" spans="1:4" ht="16" customHeight="1">
       <c r="A64" s="3">
         <v>63</v>
       </c>
       <c r="B64" s="3" t="s">
+        <v>504</v>
+      </c>
+      <c r="C64" s="3" t="s">
         <v>505</v>
       </c>
-      <c r="C64" s="3" t="s">
+      <c r="D64" s="3" t="s">
         <v>506</v>
       </c>
-      <c r="D64" s="3" t="s">
-        <v>507</v>
-      </c>
     </row>
-    <row r="65" spans="1:4" ht="16">
+    <row r="65" spans="1:4" ht="16" customHeight="1">
       <c r="A65" s="3"/>
       <c r="B65" s="3"/>
       <c r="C65" s="3"/>
       <c r="D65" s="3"/>
     </row>
-    <row r="66" spans="1:4" ht="16">
+    <row r="66" spans="1:4" ht="16" customHeight="1">
       <c r="A66" s="3"/>
       <c r="B66" s="3"/>
       <c r="C66" s="3"/>
       <c r="D66" s="3"/>
     </row>
-    <row r="67" spans="1:4" ht="16">
+    <row r="67" spans="1:4" ht="16" customHeight="1">
       <c r="A67" s="3"/>
       <c r="B67" s="3"/>
       <c r="C67" s="3"/>

</xml_diff>

<commit_message>
Mark Navon preprint as resolved in Dataset_inf.xlsx and AGENTS.md
</commit_message>
<xml_diff>
--- a/1_Data/Dataset_inf.xlsx
+++ b/1_Data/Dataset_inf.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/T3/Dell5510/HCP_cloud/My_Lab/Projects/SPE_Database/1_Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F43C018-C2EE-E646-9C67-27457FED6E61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FC653B4-E7C8-E144-B1AD-B6EF1D25CEC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="32260" yWindow="2540" windowWidth="32660" windowHeight="13940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1391" uniqueCount="516">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1391" uniqueCount="517">
   <si>
     <t>Note</t>
   </si>
@@ -1588,6 +1588,9 @@
   </si>
   <si>
     <t>http://osf.io/2q9w7</t>
+  </si>
+  <si>
+    <t>preprint</t>
   </si>
 </sst>
 </file>
@@ -1701,7 +1704,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1770,6 +1773,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -9777,8 +9783,8 @@
       <c r="L23" s="19">
         <v>2021</v>
       </c>
-      <c r="M23" s="19" t="s">
-        <v>66</v>
+      <c r="M23" s="25" t="s">
+        <v>516</v>
       </c>
       <c r="N23" s="3">
         <v>1</v>

</xml_diff>